<commit_message>
Weapon refactorisation mainly done for now. Needs to be done again to break down projectile script, but for now, in interests of progression, moving on. Now fixing bugs in current projectile behaviours
</commit_message>
<xml_diff>
--- a/SD_WorkLog.xlsx
+++ b/SD_WorkLog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adamj\Documents\Game Development\Godot\Smash Dungeon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{25AD8F85-F324-485B-BD97-63E50F936577}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{564EEED0-F28B-4C4F-87E7-87FF8ABFBE06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3120" yWindow="3120" windowWidth="21600" windowHeight="11235" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
   <si>
     <t>Smash Dungeon</t>
   </si>
@@ -63,6 +63,9 @@
   </si>
   <si>
     <t>Dev Work Log</t>
+  </si>
+  <si>
+    <t>Standardised new refactoring across all weapon behaviour. Many bugs, attempting to address bugs.</t>
   </si>
 </sst>
 </file>
@@ -149,8 +152,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="A4:E6" totalsRowShown="0">
-  <autoFilter ref="A4:E6" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="A4:E8" totalsRowShown="0">
+  <autoFilter ref="A4:E8" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{9EDA08BC-FC93-4374-BA7A-6AB42BF27608}" name="Date"/>
     <tableColumn id="2" xr3:uid="{E52E82DE-B123-4B3E-8A7E-4FB2C6CEEE64}" name="Start" dataDxfId="1"/>
@@ -479,7 +482,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F0887D6-8664-4804-98D8-EE817E3A6A1B}">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -538,6 +541,31 @@
       <c r="B6" s="2">
         <v>0.87013888888888891</v>
       </c>
+      <c r="C6" s="2">
+        <v>4.1666666666666664E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>45739</v>
+      </c>
+      <c r="B7" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="C7" s="2">
+        <v>0.5625</v>
+      </c>
+      <c r="D7" t="s">
+        <v>1</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B8" s="2">
+        <v>0.70833333333333337</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
All weapons tested and now working. Bugs fixed. Adjustments still to be considered
</commit_message>
<xml_diff>
--- a/SD_WorkLog.xlsx
+++ b/SD_WorkLog.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adamj\Documents\Game Development\Godot\Smash Dungeon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{564EEED0-F28B-4C4F-87E7-87FF8ABFBE06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77E71DCC-7BDC-4B35-981B-68E73C7B3CE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3120" yWindow="3120" windowWidth="21600" windowHeight="11235" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Smash Dungeon" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
   <si>
     <t>Smash Dungeon</t>
   </si>
@@ -66,6 +66,15 @@
   </si>
   <si>
     <t>Standardised new refactoring across all weapon behaviour. Many bugs, attempting to address bugs.</t>
+  </si>
+  <si>
+    <t>Refactoring complete (still not as refactored as much as would like as projectile.gd still handles more than I would really like, but in interest of moving forward am making do with what we have for now). Now trouble fixing bugs in how projectiles are behaving. Fixed homing, fixed cluster bomb, currently fixing bounce orb (not bouncing)</t>
+  </si>
+  <si>
+    <t>Total hours:</t>
+  </si>
+  <si>
+    <t>Time</t>
   </si>
 </sst>
 </file>
@@ -131,7 +140,10 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="3">
+    <dxf>
+      <numFmt numFmtId="25" formatCode="hh:mm"/>
+    </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -152,14 +164,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="A4:E8" totalsRowShown="0">
-  <autoFilter ref="A4:E8" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
-  <tableColumns count="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="A6:F11" totalsRowShown="0">
+  <autoFilter ref="A6:F11" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
+  <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{9EDA08BC-FC93-4374-BA7A-6AB42BF27608}" name="Date"/>
-    <tableColumn id="2" xr3:uid="{E52E82DE-B123-4B3E-8A7E-4FB2C6CEEE64}" name="Start" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{E52E82DE-B123-4B3E-8A7E-4FB2C6CEEE64}" name="Start" dataDxfId="2"/>
     <tableColumn id="3" xr3:uid="{385CF12C-F475-4237-A1B1-BA2B136D502D}" name="Finish"/>
     <tableColumn id="4" xr3:uid="{A53CF1BF-F8B6-4BD3-8E81-2C1B7E645EAD}" name="Task"/>
-    <tableColumn id="5" xr3:uid="{82A06DB5-D5A5-417C-9A3D-8CC5431A3DD7}" name="Details" dataDxfId="0"/>
+    <tableColumn id="5" xr3:uid="{82A06DB5-D5A5-417C-9A3D-8CC5431A3DD7}" name="Details" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{6B5828D5-4B73-426F-9AEB-9B2280524C8F}" name="Time" dataDxfId="0">
+      <calculatedColumnFormula>IF(C7&lt;B7, C7+1, C7) - B7</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight18" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -482,7 +497,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F0887D6-8664-4804-98D8-EE817E3A6A1B}">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -491,80 +506,135 @@
     <col min="5" max="5" width="47.42578125" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="4" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:8" s="4" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
       <c r="E1" s="5"/>
     </row>
-    <row r="2" spans="1:5" s="4" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:8" s="4" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A2" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E2" s="5"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="2">
+        <f>SUM(F7:F37)</f>
+        <v>0.5180555555555556</v>
+      </c>
+      <c r="H4" s="2"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H5" s="2"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>6</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B6" t="s">
         <v>3</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C6" t="s">
         <v>4</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D6" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E6" s="3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="1">
+      <c r="F6" t="s">
+        <v>12</v>
+      </c>
+      <c r="H6" s="2"/>
+    </row>
+    <row r="7" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
         <v>45738</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B7" s="2">
         <v>0.625</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C7" s="2">
         <v>0.77430555555555558</v>
-      </c>
-      <c r="D5" t="s">
-        <v>1</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B6" s="2">
-        <v>0.87013888888888891</v>
-      </c>
-      <c r="C6" s="2">
-        <v>4.1666666666666664E-2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="1">
-        <v>45739</v>
-      </c>
-      <c r="B7" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="C7" s="2">
-        <v>0.5625</v>
       </c>
       <c r="D7" t="s">
         <v>1</v>
       </c>
       <c r="E7" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="F7" s="2">
+        <f t="shared" ref="F7:F11" si="0">IF(C7&lt;B7, C7+1, C7) - B7</f>
+        <v>0.14930555555555558</v>
+      </c>
+      <c r="H7" s="2"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B8" s="2">
+        <v>0.87013888888888891</v>
+      </c>
+      <c r="C8" s="2">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="F8" s="2">
+        <f t="shared" si="0"/>
+        <v>0.17152777777777783</v>
+      </c>
+      <c r="H8" s="2"/>
+    </row>
+    <row r="9" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>45739</v>
+      </c>
+      <c r="B9" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="C9" s="2">
+        <v>0.5625</v>
+      </c>
+      <c r="D9" t="s">
+        <v>1</v>
+      </c>
+      <c r="E9" s="3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B8" s="2">
-        <v>0.70833333333333337</v>
+      <c r="F9" s="2">
+        <f t="shared" si="0"/>
+        <v>6.25E-2</v>
+      </c>
+      <c r="H9" s="2"/>
+    </row>
+    <row r="10" spans="1:8" ht="105" x14ac:dyDescent="0.25">
+      <c r="B10" s="2">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="C10" s="2">
+        <v>0.88472222222222219</v>
+      </c>
+      <c r="D10" t="s">
+        <v>1</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F10" s="2">
+        <f t="shared" si="0"/>
+        <v>9.3055555555555558E-2</v>
+      </c>
+      <c r="H10" s="2"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B11" s="2">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="F11" s="2">
+        <f t="shared" si="0"/>
+        <v>4.166666666666663E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
new files totally refactoring weapons system
</commit_message>
<xml_diff>
--- a/SD_WorkLog.xlsx
+++ b/SD_WorkLog.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adamj\Documents\Game Development\Godot\Smash Dungeon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77E71DCC-7BDC-4B35-981B-68E73C7B3CE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B037CD74-5A6C-4D48-BDCA-C46A72A74AF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="3120" windowWidth="21600" windowHeight="11235" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
+    <workbookView minimized="1" xWindow="3120" yWindow="3120" windowWidth="15030" windowHeight="11235" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
   </bookViews>
   <sheets>
     <sheet name="Smash Dungeon" sheetId="1" r:id="rId1"/>
+    <sheet name="Godot Learning" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="18">
   <si>
     <t>Smash Dungeon</t>
   </si>
@@ -75,6 +76,21 @@
   </si>
   <si>
     <t>Time</t>
+  </si>
+  <si>
+    <t>Fixed bugs in all projectile weapons (apart from those which are down to preference and want to make better/different)</t>
+  </si>
+  <si>
+    <t>Godot Learning</t>
+  </si>
+  <si>
+    <t>Dev Practice Log</t>
+  </si>
+  <si>
+    <t>Refactoring projectile system and improving behaviour system</t>
+  </si>
+  <si>
+    <t>Ask whether references to "improved_behaviour_manager" or just behaviour manager etc</t>
   </si>
 </sst>
 </file>
@@ -140,7 +156,16 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="6">
+    <dxf>
+      <numFmt numFmtId="25" formatCode="hh:mm"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="25" formatCode="hh:mm"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="25" formatCode="hh:mm"/>
     </dxf>
@@ -164,15 +189,32 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="A6:F11" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="A6:F12" totalsRowShown="0">
+  <autoFilter ref="A6:F12" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{9EDA08BC-FC93-4374-BA7A-6AB42BF27608}" name="Date"/>
+    <tableColumn id="2" xr3:uid="{E52E82DE-B123-4B3E-8A7E-4FB2C6CEEE64}" name="Start" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{385CF12C-F475-4237-A1B1-BA2B136D502D}" name="Finish"/>
+    <tableColumn id="4" xr3:uid="{A53CF1BF-F8B6-4BD3-8E81-2C1B7E645EAD}" name="Task"/>
+    <tableColumn id="5" xr3:uid="{82A06DB5-D5A5-417C-9A3D-8CC5431A3DD7}" name="Details" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{6B5828D5-4B73-426F-9AEB-9B2280524C8F}" name="Time" dataDxfId="3">
+      <calculatedColumnFormula>IF(C7&lt;B7, C7+1, C7) - B7</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight18" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7A4A6574-3FF0-4809-85FD-1DDCB83EA4DD}" name="Table22" displayName="Table22" ref="A6:F11" totalsRowShown="0">
   <autoFilter ref="A6:F11" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{9EDA08BC-FC93-4374-BA7A-6AB42BF27608}" name="Date"/>
-    <tableColumn id="2" xr3:uid="{E52E82DE-B123-4B3E-8A7E-4FB2C6CEEE64}" name="Start" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{385CF12C-F475-4237-A1B1-BA2B136D502D}" name="Finish"/>
-    <tableColumn id="4" xr3:uid="{A53CF1BF-F8B6-4BD3-8E81-2C1B7E645EAD}" name="Task"/>
-    <tableColumn id="5" xr3:uid="{82A06DB5-D5A5-417C-9A3D-8CC5431A3DD7}" name="Details" dataDxfId="1"/>
-    <tableColumn id="6" xr3:uid="{6B5828D5-4B73-426F-9AEB-9B2280524C8F}" name="Time" dataDxfId="0">
+    <tableColumn id="1" xr3:uid="{79650798-B691-458A-BE4A-5916DBAC4166}" name="Date"/>
+    <tableColumn id="2" xr3:uid="{064DF555-2569-4B26-8250-62634D76A69A}" name="Start" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{20620684-1ED7-4B49-B03F-DD32723B4EEF}" name="Finish"/>
+    <tableColumn id="4" xr3:uid="{82FD299F-7E84-4584-8794-9F819C3DD798}" name="Task"/>
+    <tableColumn id="5" xr3:uid="{C4AAFEC7-694F-42A2-A652-7DBB66C273C0}" name="Details" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{3FF97942-C807-4B84-B488-6C3FE6D21D35}" name="Time" dataDxfId="0">
       <calculatedColumnFormula>IF(C7&lt;B7, C7+1, C7) - B7</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -497,6 +539,184 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F0887D6-8664-4804-98D8-EE817E3A6A1B}">
+  <dimension ref="A1:L12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="10.42578125" customWidth="1"/>
+    <col min="4" max="4" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="47.42578125" style="3" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" s="4" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" s="5"/>
+    </row>
+    <row r="2" spans="1:12" s="4" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
+      <c r="A2" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="5"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="2">
+        <f>SUM(F7:F37)</f>
+        <v>1.0319444444444446</v>
+      </c>
+      <c r="H4" s="2"/>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H5" s="2"/>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D6" t="s">
+        <v>5</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F6" t="s">
+        <v>12</v>
+      </c>
+      <c r="H6" s="2"/>
+      <c r="L6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>45738</v>
+      </c>
+      <c r="B7" s="2">
+        <v>0.625</v>
+      </c>
+      <c r="C7" s="2">
+        <v>0.77430555555555558</v>
+      </c>
+      <c r="D7" t="s">
+        <v>1</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="F7" s="2">
+        <f t="shared" ref="F7:F11" si="0">IF(C7&lt;B7, C7+1, C7) - B7</f>
+        <v>0.14930555555555558</v>
+      </c>
+      <c r="H7" s="2"/>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B8" s="2">
+        <v>0.87013888888888891</v>
+      </c>
+      <c r="C8" s="2">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="F8" s="2">
+        <f t="shared" si="0"/>
+        <v>0.17152777777777783</v>
+      </c>
+      <c r="H8" s="2"/>
+    </row>
+    <row r="9" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>45739</v>
+      </c>
+      <c r="B9" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="C9" s="2">
+        <v>0.5625</v>
+      </c>
+      <c r="D9" t="s">
+        <v>1</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F9" s="2">
+        <f t="shared" si="0"/>
+        <v>6.25E-2</v>
+      </c>
+      <c r="H9" s="2"/>
+    </row>
+    <row r="10" spans="1:12" ht="105" x14ac:dyDescent="0.25">
+      <c r="B10" s="2">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="C10" s="2">
+        <v>0.88472222222222219</v>
+      </c>
+      <c r="D10" t="s">
+        <v>1</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F10" s="2">
+        <f t="shared" si="0"/>
+        <v>9.3055555555555558E-2</v>
+      </c>
+      <c r="H10" s="2"/>
+    </row>
+    <row r="11" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+      <c r="B11" s="2">
+        <v>0.97430555555555554</v>
+      </c>
+      <c r="C11" s="2">
+        <v>7.1527777777777773E-2</v>
+      </c>
+      <c r="D11" t="s">
+        <v>1</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F11" s="2">
+        <f t="shared" si="0"/>
+        <v>9.7222222222222321E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>45740</v>
+      </c>
+      <c r="B12" s="2">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F12" s="2">
+        <f>IF(C12&lt;B12, C12+1, C12) - B12</f>
+        <v>0.45833333333333337</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16EBAB43-9BF7-46C1-BE2D-33751923E718}">
   <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -508,13 +728,13 @@
   <sheetData>
     <row r="1" spans="1:8" s="4" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A1" s="4" t="s">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="E1" s="5"/>
     </row>
     <row r="2" spans="1:8" s="4" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A2" s="6" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="E2" s="5"/>
     </row>
@@ -524,7 +744,7 @@
       </c>
       <c r="C4" s="2">
         <f>SUM(F7:F37)</f>
-        <v>0.5180555555555556</v>
+        <v>0</v>
       </c>
       <c r="H4" s="2"/>
     </row>
@@ -552,89 +772,50 @@
       </c>
       <c r="H6" s="2"/>
     </row>
-    <row r="7" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="1">
-        <v>45738</v>
-      </c>
-      <c r="B7" s="2">
-        <v>0.625</v>
-      </c>
-      <c r="C7" s="2">
-        <v>0.77430555555555558</v>
-      </c>
-      <c r="D7" t="s">
-        <v>1</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>2</v>
-      </c>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="1"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
       <c r="F7" s="2">
         <f t="shared" ref="F7:F11" si="0">IF(C7&lt;B7, C7+1, C7) - B7</f>
-        <v>0.14930555555555558</v>
+        <v>0</v>
       </c>
       <c r="H7" s="2"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B8" s="2">
-        <v>0.87013888888888891</v>
-      </c>
-      <c r="C8" s="2">
-        <v>4.1666666666666664E-2</v>
-      </c>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
       <c r="F8" s="2">
         <f t="shared" si="0"/>
-        <v>0.17152777777777783</v>
+        <v>0</v>
       </c>
       <c r="H8" s="2"/>
     </row>
-    <row r="9" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A9" s="1">
-        <v>45739</v>
-      </c>
-      <c r="B9" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="C9" s="2">
-        <v>0.5625</v>
-      </c>
-      <c r="D9" t="s">
-        <v>1</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>9</v>
-      </c>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="1"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
       <c r="F9" s="2">
         <f t="shared" si="0"/>
-        <v>6.25E-2</v>
+        <v>0</v>
       </c>
       <c r="H9" s="2"/>
     </row>
-    <row r="10" spans="1:8" ht="105" x14ac:dyDescent="0.25">
-      <c r="B10" s="2">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="C10" s="2">
-        <v>0.88472222222222219</v>
-      </c>
-      <c r="D10" t="s">
-        <v>1</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>10</v>
-      </c>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
       <c r="F10" s="2">
         <f t="shared" si="0"/>
-        <v>9.3055555555555558E-2</v>
+        <v>0</v>
       </c>
       <c r="H10" s="2"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B11" s="2">
-        <v>0.95833333333333337</v>
-      </c>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
       <c r="F11" s="2">
         <f t="shared" si="0"/>
-        <v>4.166666666666663E-2</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactor complete. Bug fixing weapons now
</commit_message>
<xml_diff>
--- a/SD_WorkLog.xlsx
+++ b/SD_WorkLog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adamj\Documents\Game Development\Godot\Smash Dungeon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B037CD74-5A6C-4D48-BDCA-C46A72A74AF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD392ED7-29D1-41E9-A67D-20A1E721591D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="3120" yWindow="3120" windowWidth="15030" windowHeight="11235" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
   </bookViews>
   <sheets>
     <sheet name="Smash Dungeon" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="20">
   <si>
     <t>Smash Dungeon</t>
   </si>
@@ -91,6 +91,17 @@
   </si>
   <si>
     <t>Ask whether references to "improved_behaviour_manager" or just behaviour manager etc</t>
+  </si>
+  <si>
+    <t>Brackeys Tutorial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Starting from scratch
+- animatable body2d (for moving objects you want to collide with, e.g. platform)
+- enabled one-way collision in transport so player can jump from below
+- animated spite2d (for player character)
+-collision shape 2d (for player collision)
+</t>
   </si>
 </sst>
 </file>
@@ -566,7 +577,7 @@
       </c>
       <c r="C4" s="2">
         <f>SUM(F7:F37)</f>
-        <v>1.0319444444444446</v>
+        <v>0.71944444444444466</v>
       </c>
       <c r="H4" s="2"/>
     </row>
@@ -698,12 +709,15 @@
       <c r="B12" s="2">
         <v>0.54166666666666663</v>
       </c>
+      <c r="C12" s="2">
+        <v>0.6875</v>
+      </c>
       <c r="E12" s="3" t="s">
         <v>16</v>
       </c>
       <c r="F12" s="2">
         <f>IF(C12&lt;B12, C12+1, C12) - B12</f>
-        <v>0.45833333333333337</v>
+        <v>0.14583333333333337</v>
       </c>
     </row>
   </sheetData>
@@ -744,7 +758,7 @@
       </c>
       <c r="C4" s="2">
         <f>SUM(F7:F37)</f>
-        <v>0</v>
+        <v>2.083333333333337E-2</v>
       </c>
       <c r="H4" s="2"/>
     </row>
@@ -772,13 +786,25 @@
       </c>
       <c r="H6" s="2"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="1"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
+    <row r="7" spans="1:8" ht="120" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>45740</v>
+      </c>
+      <c r="B7" s="2">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="C7" s="2">
+        <v>0.9375</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="F7" s="2">
         <f t="shared" ref="F7:F11" si="0">IF(C7&lt;B7, C7+1, C7) - B7</f>
-        <v>0</v>
+        <v>2.083333333333337E-2</v>
       </c>
       <c r="H7" s="2"/>
     </row>

</xml_diff>

<commit_message>
fixing physics and movement
</commit_message>
<xml_diff>
--- a/SD_WorkLog.xlsx
+++ b/SD_WorkLog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adamj\Documents\Game Development\Godot\Smash Dungeon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD392ED7-29D1-41E9-A67D-20A1E721591D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{163803CD-1F74-4B04-BAE8-186E10E3627F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="20">
   <si>
     <t>Smash Dungeon</t>
   </si>
@@ -88,9 +88,6 @@
   </si>
   <si>
     <t>Refactoring projectile system and improving behaviour system</t>
-  </si>
-  <si>
-    <t>Ask whether references to "improved_behaviour_manager" or just behaviour manager etc</t>
   </si>
   <si>
     <t>Brackeys Tutorial</t>
@@ -102,6 +99,10 @@
 - animated spite2d (for player character)
 -collision shape 2d (for player collision)
 </t>
+  </si>
+  <si>
+    <t>Refactoring system complete. Bug fixes for weapons.
+Annoying 'indent' issue, hoping just needed a close and restart, will test tomorrow.</t>
   </si>
 </sst>
 </file>
@@ -200,8 +201,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="A6:F12" totalsRowShown="0">
-  <autoFilter ref="A6:F12" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="A6:F13" totalsRowShown="0">
+  <autoFilter ref="A6:F13" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{9EDA08BC-FC93-4374-BA7A-6AB42BF27608}" name="Date"/>
     <tableColumn id="2" xr3:uid="{E52E82DE-B123-4B3E-8A7E-4FB2C6CEEE64}" name="Start" dataDxfId="5"/>
@@ -550,7 +551,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F0887D6-8664-4804-98D8-EE817E3A6A1B}">
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -559,32 +560,32 @@
     <col min="5" max="5" width="47.42578125" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="4" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:8" s="4" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
       <c r="E1" s="5"/>
     </row>
-    <row r="2" spans="1:12" s="4" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:8" s="4" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A2" s="6" t="s">
         <v>8</v>
       </c>
       <c r="E2" s="5"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>11</v>
       </c>
       <c r="C4" s="2">
         <f>SUM(F7:F37)</f>
-        <v>0.71944444444444466</v>
+        <v>0.7958333333333335</v>
       </c>
       <c r="H4" s="2"/>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H5" s="2"/>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -604,11 +605,8 @@
         <v>12</v>
       </c>
       <c r="H6" s="2"/>
-      <c r="L6" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>45738</v>
       </c>
@@ -630,7 +628,7 @@
       </c>
       <c r="H7" s="2"/>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B8" s="2">
         <v>0.87013888888888891</v>
       </c>
@@ -643,7 +641,7 @@
       </c>
       <c r="H8" s="2"/>
     </row>
-    <row r="9" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>45739</v>
       </c>
@@ -665,7 +663,7 @@
       </c>
       <c r="H9" s="2"/>
     </row>
-    <row r="10" spans="1:12" ht="105" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" ht="105" x14ac:dyDescent="0.25">
       <c r="B10" s="2">
         <v>0.79166666666666663</v>
       </c>
@@ -684,7 +682,7 @@
       </c>
       <c r="H10" s="2"/>
     </row>
-    <row r="11" spans="1:12" ht="45" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="B11" s="2">
         <v>0.97430555555555554</v>
       </c>
@@ -702,7 +700,7 @@
         <v>9.7222222222222321E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>45740</v>
       </c>
@@ -711,6 +709,9 @@
       </c>
       <c r="C12" s="2">
         <v>0.6875</v>
+      </c>
+      <c r="D12" t="s">
+        <v>1</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>16</v>
@@ -718,6 +719,24 @@
       <c r="F12" s="2">
         <f>IF(C12&lt;B12, C12+1, C12) - B12</f>
         <v>0.14583333333333337</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="B13" s="2">
+        <v>0.98611111111111116</v>
+      </c>
+      <c r="C13" s="2">
+        <v>6.25E-2</v>
+      </c>
+      <c r="D13" t="s">
+        <v>1</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F13" s="2">
+        <f>IF(C13&lt;B13, C13+1, C13) - B13</f>
+        <v>7.638888888888884E-2</v>
       </c>
     </row>
   </sheetData>
@@ -797,10 +816,10 @@
         <v>0.9375</v>
       </c>
       <c r="D7" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7" s="3" t="s">
         <v>18</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>19</v>
       </c>
       <c r="F7" s="2">
         <f t="shared" ref="F7:F11" si="0">IF(C7&lt;B7, C7+1, C7) - B7</f>

</xml_diff>

<commit_message>
Cleaned up weapon system. Now moving on to fixing all weapon behaviors
</commit_message>
<xml_diff>
--- a/SD_WorkLog.xlsx
+++ b/SD_WorkLog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adamj\Documents\Game Development\Godot\Smash Dungeon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{163803CD-1F74-4B04-BAE8-186E10E3627F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{893C9328-9735-4328-8EAD-02A688DA494A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="22">
   <si>
     <t>Smash Dungeon</t>
   </si>
@@ -104,11 +104,24 @@
     <t>Refactoring system complete. Bug fixes for weapons.
 Annoying 'indent' issue, hoping just needed a close and restart, will test tomorrow.</t>
   </si>
+  <si>
+    <t>Cleaning up refactored system.
+- Added null refernces to behaviour manager
+- Addressing missed signal connections
+- Addressing timer managerment problems
+- Physics and movement issues</t>
+  </si>
+  <si>
+    <t>Fixing bugs with all weapons. Not very happy with how much weapons have all changed, but hopefully continual bug fixing will end up with a more resiliant system once done.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="[h]:mm"/>
+  </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -152,7 +165,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -164,6 +177,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -201,8 +215,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="A6:F13" totalsRowShown="0">
-  <autoFilter ref="A6:F13" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G15" totalsRowShown="0">
+  <autoFilter ref="B6:G15" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{9EDA08BC-FC93-4374-BA7A-6AB42BF27608}" name="Date"/>
     <tableColumn id="2" xr3:uid="{E52E82DE-B123-4B3E-8A7E-4FB2C6CEEE64}" name="Start" dataDxfId="5"/>
@@ -210,7 +224,7 @@
     <tableColumn id="4" xr3:uid="{A53CF1BF-F8B6-4BD3-8E81-2C1B7E645EAD}" name="Task"/>
     <tableColumn id="5" xr3:uid="{82A06DB5-D5A5-417C-9A3D-8CC5431A3DD7}" name="Details" dataDxfId="4"/>
     <tableColumn id="6" xr3:uid="{6B5828D5-4B73-426F-9AEB-9B2280524C8F}" name="Time" dataDxfId="3">
-      <calculatedColumnFormula>IF(C7&lt;B7, C7+1, C7) - B7</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(D7&lt;C7, D7+1, D7) - C7</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight18" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -551,192 +565,231 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F0887D6-8664-4804-98D8-EE817E3A6A1B}">
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="10.42578125" customWidth="1"/>
-    <col min="4" max="4" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="47.42578125" style="3" customWidth="1"/>
+    <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="10.42578125" customWidth="1"/>
+    <col min="5" max="5" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="47.42578125" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="4" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:9" s="4" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="5"/>
-    </row>
-    <row r="2" spans="1:8" s="4" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
+      <c r="F1" s="5"/>
+    </row>
+    <row r="2" spans="1:9" s="4" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A2" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="5"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B4" t="s">
+      <c r="F2" s="5"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C4" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="2">
-        <f>SUM(F7:F37)</f>
-        <v>0.7958333333333335</v>
-      </c>
-      <c r="H4" s="2"/>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="H5" s="2"/>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="D4" s="7">
+        <f>SUM(G7:G37)</f>
+        <v>1.0319444444444446</v>
+      </c>
+      <c r="I4" s="2"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I5" s="2"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
         <v>6</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>3</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>4</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>5</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="F6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>12</v>
       </c>
-      <c r="H6" s="2"/>
-    </row>
-    <row r="7" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="1">
+      <c r="I6" s="2"/>
+    </row>
+    <row r="7" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="B7" s="1">
         <v>45738</v>
       </c>
-      <c r="B7" s="2">
+      <c r="C7" s="2">
         <v>0.625</v>
       </c>
-      <c r="C7" s="2">
+      <c r="D7" s="2">
         <v>0.77430555555555558</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>1</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="F7" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="F7" s="2">
-        <f t="shared" ref="F7:F11" si="0">IF(C7&lt;B7, C7+1, C7) - B7</f>
+      <c r="G7" s="2">
+        <f t="shared" ref="G7:G11" si="0">IF(D7&lt;C7, D7+1, D7) - C7</f>
         <v>0.14930555555555558</v>
       </c>
-      <c r="H7" s="2"/>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B8" s="2">
+      <c r="I7" s="2"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C8" s="2">
         <v>0.87013888888888891</v>
       </c>
-      <c r="C8" s="2">
+      <c r="D8" s="2">
         <v>4.1666666666666664E-2</v>
       </c>
-      <c r="F8" s="2">
+      <c r="G8" s="2">
         <f t="shared" si="0"/>
         <v>0.17152777777777783</v>
       </c>
-      <c r="H8" s="2"/>
-    </row>
-    <row r="9" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A9" s="1">
+      <c r="I8" s="2"/>
+    </row>
+    <row r="9" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="B9" s="1">
         <v>45739</v>
       </c>
-      <c r="B9" s="2">
+      <c r="C9" s="2">
         <v>0.5</v>
       </c>
-      <c r="C9" s="2">
+      <c r="D9" s="2">
         <v>0.5625</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>1</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="F9" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="F9" s="2">
+      <c r="G9" s="2">
         <f t="shared" si="0"/>
         <v>6.25E-2</v>
       </c>
-      <c r="H9" s="2"/>
-    </row>
-    <row r="10" spans="1:8" ht="105" x14ac:dyDescent="0.25">
-      <c r="B10" s="2">
+      <c r="I9" s="2"/>
+    </row>
+    <row r="10" spans="1:9" ht="105" x14ac:dyDescent="0.25">
+      <c r="C10" s="2">
         <v>0.79166666666666663</v>
       </c>
-      <c r="C10" s="2">
+      <c r="D10" s="2">
         <v>0.88472222222222219</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
         <v>1</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="F10" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F10" s="2">
+      <c r="G10" s="2">
         <f t="shared" si="0"/>
         <v>9.3055555555555558E-2</v>
       </c>
-      <c r="H10" s="2"/>
-    </row>
-    <row r="11" spans="1:8" ht="45" x14ac:dyDescent="0.25">
-      <c r="B11" s="2">
+      <c r="I10" s="2"/>
+    </row>
+    <row r="11" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="C11" s="2">
         <v>0.97430555555555554</v>
       </c>
-      <c r="C11" s="2">
+      <c r="D11" s="2">
         <v>7.1527777777777773E-2</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>1</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="F11" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="F11" s="2">
+      <c r="G11" s="2">
         <f t="shared" si="0"/>
         <v>9.7222222222222321E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A12" s="1">
+    <row r="12" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="B12" s="1">
         <v>45740</v>
       </c>
-      <c r="B12" s="2">
+      <c r="C12" s="2">
         <v>0.54166666666666663</v>
       </c>
-      <c r="C12" s="2">
+      <c r="D12" s="2">
         <v>0.6875</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>1</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="F12" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="F12" s="2">
-        <f>IF(C12&lt;B12, C12+1, C12) - B12</f>
+      <c r="G12" s="2">
+        <f>IF(D12&lt;C12, D12+1, D12) - C12</f>
         <v>0.14583333333333337</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="60" x14ac:dyDescent="0.25">
-      <c r="B13" s="2">
+    <row r="13" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="C13" s="2">
         <v>0.98611111111111116</v>
       </c>
-      <c r="C13" s="2">
+      <c r="D13" s="2">
         <v>6.25E-2</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E13" t="s">
         <v>1</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="F13" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="F13" s="2">
-        <f>IF(C13&lt;B13, C13+1, C13) - B13</f>
+      <c r="G13" s="2">
+        <f>IF(D13&lt;C13, D13+1, D13) - C13</f>
         <v>7.638888888888884E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+      <c r="B14" s="1">
+        <v>45741</v>
+      </c>
+      <c r="C14" s="2">
+        <v>0.63888888888888884</v>
+      </c>
+      <c r="D14" s="2">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="E14" t="s">
+        <v>1</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G14" s="2">
+        <f>IF(D14&lt;C14, D14+1, D14) - C14</f>
+        <v>0.15277777777777779</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="C15" s="2">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="D15" s="2">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="E15" t="s">
+        <v>1</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="G15" s="2">
+        <f>IF(D15&lt;C15, D15+1, D15) - C15</f>
+        <v>8.3333333333333259E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed weapon system, working on fixing data pull from csv file
</commit_message>
<xml_diff>
--- a/SD_WorkLog.xlsx
+++ b/SD_WorkLog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adamj\Documents\Game Development\Godot\Smash Dungeon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{893C9328-9735-4328-8EAD-02A688DA494A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F371EE69-A42B-426C-8C55-77087561231B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="23">
   <si>
     <t>Smash Dungeon</t>
   </si>
@@ -114,13 +114,20 @@
   <si>
     <t>Fixing bugs with all weapons. Not very happy with how much weapons have all changed, but hopefully continual bug fixing will end up with a more resiliant system once done.</t>
   </si>
+  <si>
+    <t>Tidied up the following:
+- Fixed Signal Safety Issues – Ensured all signals were properly connected and disconnected. 
+- Fixed Behavior Application – Made sure behaviors were correctly applied to projectiles. 
+- Implemented Safe Metadata Access – Added checks before accessing metadata.
+- Added Null Reference Checks – Protected against null reference exceptions.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="[h]:mm"/>
+    <numFmt numFmtId="164" formatCode="[h]:mm"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -177,7 +184,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -215,8 +222,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G15" totalsRowShown="0">
-  <autoFilter ref="B6:G15" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G20" totalsRowShown="0">
+  <autoFilter ref="B6:G20" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{9EDA08BC-FC93-4374-BA7A-6AB42BF27608}" name="Date"/>
     <tableColumn id="2" xr3:uid="{E52E82DE-B123-4B3E-8A7E-4FB2C6CEEE64}" name="Start" dataDxfId="5"/>
@@ -565,7 +572,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F0887D6-8664-4804-98D8-EE817E3A6A1B}">
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -591,8 +598,8 @@
         <v>11</v>
       </c>
       <c r="D4" s="7">
-        <f>SUM(G7:G37)</f>
-        <v>1.0319444444444446</v>
+        <f>SUM(G7:G41)</f>
+        <v>1.1361111111111111</v>
       </c>
       <c r="I4" s="2"/>
     </row>
@@ -790,6 +797,63 @@
       <c r="G15" s="2">
         <f>IF(D15&lt;C15, D15+1, D15) - C15</f>
         <v>8.3333333333333259E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="135" x14ac:dyDescent="0.25">
+      <c r="B16" s="1">
+        <v>45742</v>
+      </c>
+      <c r="C16" s="2">
+        <v>0.6875</v>
+      </c>
+      <c r="D16" s="2">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="E16" t="s">
+        <v>1</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G16" s="2">
+        <f>IF(D16&lt;C16, D16+1, D16) - C16</f>
+        <v>0.10416666666666663</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B17" s="1"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+      <c r="G17" s="2">
+        <f t="shared" ref="G17:G20" si="1">IF(D17&lt;C17, D17+1, D17) - C17</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B18" s="1"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="G18" s="2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B19" s="1"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="G19" s="2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B20" s="1"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
+      <c r="G20" s="2">
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed singularity, trying to fix cluster bomb and multi staff
</commit_message>
<xml_diff>
--- a/SD_WorkLog.xlsx
+++ b/SD_WorkLog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adamj\Documents\Game Development\Godot\Smash Dungeon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F371EE69-A42B-426C-8C55-77087561231B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A65E6C48-1CDC-4150-BD80-A1BB4AFB5C49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="25">
   <si>
     <t>Smash Dungeon</t>
   </si>
@@ -120,6 +120,15 @@
 - Fixed Behavior Application – Made sure behaviors were correctly applied to projectiles. 
 - Implemented Safe Metadata Access – Added checks before accessing metadata.
 - Added Null Reference Checks – Protected against null reference exceptions.</t>
+  </si>
+  <si>
+    <t>Fixing singularity bomb</t>
+  </si>
+  <si>
+    <t>Fixed singularity
+Fixed bounce orb
+Added wild bounce orb
+Started working on cluster bomb</t>
   </si>
 </sst>
 </file>
@@ -599,7 +608,7 @@
       </c>
       <c r="D4" s="7">
         <f>SUM(G7:G41)</f>
-        <v>1.1361111111111111</v>
+        <v>1.6152777777777776</v>
       </c>
       <c r="I4" s="2"/>
     </row>
@@ -821,30 +830,64 @@
       </c>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B17" s="1"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
+      <c r="B17" s="1">
+        <v>45744</v>
+      </c>
+      <c r="C17" s="2">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="D17" s="2">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="E17" t="s">
+        <v>1</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>23</v>
+      </c>
       <c r="G17" s="2">
         <f t="shared" ref="G17:G20" si="1">IF(D17&lt;C17, D17+1, D17) - C17</f>
-        <v>0</v>
+        <v>0.25000000000000011</v>
       </c>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B18" s="1"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
+      <c r="B18" s="1">
+        <v>45745</v>
+      </c>
+      <c r="C18" s="2">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="D18" s="2">
+        <v>0.52083333333333337</v>
+      </c>
+      <c r="E18" t="s">
+        <v>1</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>23</v>
+      </c>
       <c r="G18" s="2">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
+        <v>6.2500000000000056E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7" ht="60" x14ac:dyDescent="0.25">
       <c r="B19" s="1"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
+      <c r="C19" s="2">
+        <v>0.625</v>
+      </c>
+      <c r="D19" s="2">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="E19" t="s">
+        <v>1</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>24</v>
+      </c>
       <c r="G19" s="2">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.16666666666666663</v>
       </c>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Separated new behaviors, now trying to parse them with behavior manager
</commit_message>
<xml_diff>
--- a/SD_WorkLog.xlsx
+++ b/SD_WorkLog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adamj\Documents\Game Development\Godot\Smash Dungeon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A65E6C48-1CDC-4150-BD80-A1BB4AFB5C49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC31BCD0-4908-46ED-BA7D-6135842E7A8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="27">
   <si>
     <t>Smash Dungeon</t>
   </si>
@@ -129,6 +129,16 @@
 Fixed bounce orb
 Added wild bounce orb
 Started working on cluster bomb</t>
+  </si>
+  <si>
+    <t>Fixing cluster bomb</t>
+  </si>
+  <si>
+    <t>Fixing cluster bomb
+- created new cluster bomb behavior
+- created new arc behavior
+- created new explosion behavior
+- created new multishot behavior</t>
   </si>
 </sst>
 </file>
@@ -231,8 +241,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G20" totalsRowShown="0">
-  <autoFilter ref="B6:G20" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G22" totalsRowShown="0">
+  <autoFilter ref="B6:G22" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{9EDA08BC-FC93-4374-BA7A-6AB42BF27608}" name="Date"/>
     <tableColumn id="2" xr3:uid="{E52E82DE-B123-4B3E-8A7E-4FB2C6CEEE64}" name="Start" dataDxfId="5"/>
@@ -581,7 +591,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F0887D6-8664-4804-98D8-EE817E3A6A1B}">
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -608,7 +618,7 @@
       </c>
       <c r="D4" s="7">
         <f>SUM(G7:G41)</f>
-        <v>1.6152777777777776</v>
+        <v>2.34375</v>
       </c>
       <c r="I4" s="2"/>
     </row>
@@ -892,11 +902,54 @@
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B20" s="1"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
+      <c r="C20" s="2">
+        <v>0.875</v>
+      </c>
+      <c r="D20" s="2">
+        <v>0.4375</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>25</v>
+      </c>
       <c r="G20" s="2">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.5625</v>
+      </c>
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C21" s="2">
+        <v>0.98958333333333337</v>
+      </c>
+      <c r="D21" s="2">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G21" s="2">
+        <f>IF(D21&lt;C21, D21+1, D21) - C21</f>
+        <v>5.208333333333337E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="2:7" ht="75" x14ac:dyDescent="0.25">
+      <c r="B22" s="1">
+        <v>45746</v>
+      </c>
+      <c r="C22" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="D22" s="2">
+        <v>0.61388888888888893</v>
+      </c>
+      <c r="E22" t="s">
+        <v>1</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G22" s="2">
+        <f>IF(D22&lt;C22, D22+1, D22) - C22</f>
+        <v>0.11388888888888893</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed new bexier behavior and cluster bomb
</commit_message>
<xml_diff>
--- a/SD_WorkLog.xlsx
+++ b/SD_WorkLog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adamj\Documents\Game Development\Godot\Smash Dungeon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC31BCD0-4908-46ED-BA7D-6135842E7A8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F1EFB10-DFDA-4B58-B3A6-99035AE40B27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
+    <workbookView xWindow="3465" yWindow="3465" windowWidth="21600" windowHeight="11235" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
   </bookViews>
   <sheets>
     <sheet name="Smash Dungeon" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="30">
   <si>
     <t>Smash Dungeon</t>
   </si>
@@ -139,6 +139,20 @@
 - created new arc behavior
 - created new explosion behavior
 - created new multishot behavior</t>
+  </si>
+  <si>
+    <t>Trying to fix behavior manager to parse new behaviors</t>
+  </si>
+  <si>
+    <t>Tried using bezier behavior instead of arc for falling curve
+- Created new BezierBehavior
+- Updated multishot to try to give individual arcs
+- Troubleshooting bezier behavior</t>
+  </si>
+  <si>
+    <t>Fixed Cluster bomb/bezier behavior
+- exploring how to adjust parameters in script
+- question over how these changes to parameters could be utilised in weapon data</t>
   </si>
 </sst>
 </file>
@@ -241,8 +255,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G22" totalsRowShown="0">
-  <autoFilter ref="B6:G22" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G25" totalsRowShown="0">
+  <autoFilter ref="B6:G25" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{9EDA08BC-FC93-4374-BA7A-6AB42BF27608}" name="Date"/>
     <tableColumn id="2" xr3:uid="{E52E82DE-B123-4B3E-8A7E-4FB2C6CEEE64}" name="Start" dataDxfId="5"/>
@@ -591,7 +605,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F0887D6-8664-4804-98D8-EE817E3A6A1B}">
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -618,7 +632,7 @@
       </c>
       <c r="D4" s="7">
         <f>SUM(G7:G41)</f>
-        <v>2.34375</v>
+        <v>2.5347222222222223</v>
       </c>
       <c r="I4" s="2"/>
     </row>
@@ -950,6 +964,60 @@
       <c r="G22" s="2">
         <f>IF(D22&lt;C22, D22+1, D22) - C22</f>
         <v>0.11388888888888893</v>
+      </c>
+    </row>
+    <row r="23" spans="2:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="C23" s="2">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="D23" s="2">
+        <v>0.85763888888888884</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G23" s="2">
+        <f>IF(D23&lt;C23, D23+1, D23) - C23</f>
+        <v>6.597222222222221E-2</v>
+      </c>
+    </row>
+    <row r="24" spans="2:7" ht="75" x14ac:dyDescent="0.25">
+      <c r="B24" s="1">
+        <v>45747</v>
+      </c>
+      <c r="C24" s="2">
+        <v>0.57291666666666663</v>
+      </c>
+      <c r="D24" s="2">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="E24" t="s">
+        <v>1</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="G24" s="2">
+        <f>IF(D24&lt;C24, D24+1, D24) - C24</f>
+        <v>9.375E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="2:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="C25" s="2">
+        <v>0.75902777777777775</v>
+      </c>
+      <c r="D25" s="2">
+        <v>0.79027777777777775</v>
+      </c>
+      <c r="E25" t="s">
+        <v>1</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G25" s="2">
+        <f>IF(D25&lt;C25, D25+1, D25) - C25</f>
+        <v>3.125E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed most weapons - Singularity again needs fix
</commit_message>
<xml_diff>
--- a/SD_WorkLog.xlsx
+++ b/SD_WorkLog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adamj\Documents\Game Development\Godot\Smash Dungeon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{596AAB39-DB6D-467A-BB4B-5AF3CC8DBBAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2C508A0-34E2-465D-9D10-4EB3ACF03866}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3465" yWindow="3465" windowWidth="21600" windowHeight="11235" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
   </bookViews>
   <sheets>
     <sheet name="Smash Dungeon" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="34">
   <si>
     <t>Smash Dungeon</t>
   </si>
@@ -162,6 +162,14 @@
   </si>
   <si>
     <t>Attempting to fix shotgun</t>
+  </si>
+  <si>
+    <t>Fixed shotgun and tested most weapons
+- Need to re-fix singularity after adding bexier arc
+- Most weapons functioning
+- Need more differentation (although perhaps damage stats will help)
+- Need to build documentation to detail parameters and how to change them
+- Potentially try adding more new behaviors</t>
   </si>
 </sst>
 </file>
@@ -641,7 +649,7 @@
       </c>
       <c r="D4" s="7">
         <f>SUM(G7:G41)</f>
-        <v>2.7256944444444446</v>
+        <v>2.7631944444444443</v>
       </c>
       <c r="I4" s="2"/>
     </row>
@@ -1086,22 +1094,25 @@
         <v>3.472222222222221E-2</v>
       </c>
     </row>
-    <row r="29" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:7" ht="120" x14ac:dyDescent="0.25">
       <c r="B29" s="1">
         <v>45750</v>
       </c>
       <c r="C29" s="2">
         <v>0.96180555555555558</v>
       </c>
+      <c r="D29" s="2">
+        <v>3.7499999999999999E-2</v>
+      </c>
       <c r="E29" t="s">
         <v>1</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G29" s="2">
         <f>IF(D29&lt;C29, D29+1, D29) - C29</f>
-        <v>3.819444444444442E-2</v>
+        <v>7.5694444444444509E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added dagger attack style and started cooldown system
</commit_message>
<xml_diff>
--- a/SD_WorkLog.xlsx
+++ b/SD_WorkLog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adamj\Documents\Game Development\Godot\Smash Dungeon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2C508A0-34E2-465D-9D10-4EB3ACF03866}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5793A7E4-9776-4624-AA2E-FC4543E4D2B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="36">
   <si>
     <t>Smash Dungeon</t>
   </si>
@@ -164,12 +164,19 @@
     <t>Attempting to fix shotgun</t>
   </si>
   <si>
+    <t>Fixed Singularity
+- Fixed pull blade</t>
+  </si>
+  <si>
     <t>Fixed shotgun and tested most weapons
-- Need to re-fix singularity after adding bexier arc
+- Need to re-fix singularity after adding bezier arc
 - Most weapons functioning
 - Need more differentation (although perhaps damage stats will help)
 - Need to build documentation to detail parameters and how to change them
 - Potentially try adding more new behaviors</t>
+  </si>
+  <si>
+    <t>Added 'dagger' attack style, and started implementing 'cooldown' behavior, with meter. But cooldown and next attack don't quite seem in-line. Want to find way to make input more immediate, natural</t>
   </si>
 </sst>
 </file>
@@ -272,8 +279,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G29" totalsRowShown="0">
-  <autoFilter ref="B6:G29" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G31" totalsRowShown="0">
+  <autoFilter ref="B6:G31" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{9EDA08BC-FC93-4374-BA7A-6AB42BF27608}" name="Date"/>
     <tableColumn id="2" xr3:uid="{E52E82DE-B123-4B3E-8A7E-4FB2C6CEEE64}" name="Start" dataDxfId="5"/>
@@ -622,7 +629,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F0887D6-8664-4804-98D8-EE817E3A6A1B}">
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -649,7 +656,7 @@
       </c>
       <c r="D4" s="7">
         <f>SUM(G7:G41)</f>
-        <v>2.7631944444444443</v>
+        <v>2.8319444444444444</v>
       </c>
       <c r="I4" s="2"/>
     </row>
@@ -1108,11 +1115,50 @@
         <v>1</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G29" s="2">
         <f>IF(D29&lt;C29, D29+1, D29) - C29</f>
         <v>7.5694444444444509E-2</v>
+      </c>
+    </row>
+    <row r="30" spans="2:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="B30" s="1">
+        <v>45751</v>
+      </c>
+      <c r="C30" s="2">
+        <v>0.6875</v>
+      </c>
+      <c r="D30" s="2">
+        <v>0.72569444444444442</v>
+      </c>
+      <c r="E30" t="s">
+        <v>1</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G30" s="2">
+        <f>IF(D30&lt;C30, D30+1, D30) - C30</f>
+        <v>3.819444444444442E-2</v>
+      </c>
+    </row>
+    <row r="31" spans="2:7" ht="75" x14ac:dyDescent="0.25">
+      <c r="C31" s="2">
+        <v>0.88124999999999998</v>
+      </c>
+      <c r="D31" s="2">
+        <v>0.91180555555555554</v>
+      </c>
+      <c r="E31" t="s">
+        <v>1</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G31" s="2">
+        <f>IF(D31&lt;C31, D31+1, D31) - C31</f>
+        <v>3.0555555555555558E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
saving before updating cooldown
</commit_message>
<xml_diff>
--- a/SD_WorkLog.xlsx
+++ b/SD_WorkLog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adamj\Documents\Game Development\Godot\Smash Dungeon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5793A7E4-9776-4624-AA2E-FC4543E4D2B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D50B785D-F2AD-4D3D-BEFC-44301D603F4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="37">
   <si>
     <t>Smash Dungeon</t>
   </si>
@@ -177,6 +177,9 @@
   </si>
   <si>
     <t>Added 'dagger' attack style, and started implementing 'cooldown' behavior, with meter. But cooldown and next attack don't quite seem in-line. Want to find way to make input more immediate, natural</t>
+  </si>
+  <si>
+    <t>Fixing cooldown</t>
   </si>
 </sst>
 </file>
@@ -279,8 +282,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G31" totalsRowShown="0">
-  <autoFilter ref="B6:G31" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G32" totalsRowShown="0">
+  <autoFilter ref="B6:G32" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{9EDA08BC-FC93-4374-BA7A-6AB42BF27608}" name="Date"/>
     <tableColumn id="2" xr3:uid="{E52E82DE-B123-4B3E-8A7E-4FB2C6CEEE64}" name="Start" dataDxfId="5"/>
@@ -629,7 +632,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F0887D6-8664-4804-98D8-EE817E3A6A1B}">
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -656,7 +659,7 @@
       </c>
       <c r="D4" s="7">
         <f>SUM(G7:G41)</f>
-        <v>2.8319444444444444</v>
+        <v>3.2833333333333332</v>
       </c>
       <c r="I4" s="2"/>
     </row>
@@ -1159,6 +1162,24 @@
       <c r="G31" s="2">
         <f>IF(D31&lt;C31, D31+1, D31) - C31</f>
         <v>3.0555555555555558E-2</v>
+      </c>
+    </row>
+    <row r="32" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B32" s="1">
+        <v>45752</v>
+      </c>
+      <c r="C32" s="2">
+        <v>0.54861111111111116</v>
+      </c>
+      <c r="E32" t="s">
+        <v>1</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="G32" s="2">
+        <f>IF(D32&lt;C32, D32+1, D32) - C32</f>
+        <v>0.45138888888888884</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed weapon cooldown, but now causing some issues with weapons
</commit_message>
<xml_diff>
--- a/SD_WorkLog.xlsx
+++ b/SD_WorkLog.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adamj\Documents\Game Development\Godot\Smash Dungeon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D50B785D-F2AD-4D3D-BEFC-44301D603F4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78873092-0864-4483-A329-02093806C1A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
+    <workbookView xWindow="1560" yWindow="735" windowWidth="21600" windowHeight="11235" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
   </bookViews>
   <sheets>
     <sheet name="Smash Dungeon" sheetId="1" r:id="rId1"/>
-    <sheet name="Godot Learning" sheetId="2" r:id="rId2"/>
+    <sheet name="Card Combiner" sheetId="3" r:id="rId2"/>
+    <sheet name="Godot Learning" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="41">
   <si>
     <t>Smash Dungeon</t>
   </si>
@@ -180,6 +181,22 @@
   </si>
   <si>
     <t>Fixing cooldown</t>
+  </si>
+  <si>
+    <t>Card Combiner</t>
+  </si>
+  <si>
+    <t>Basic Mechanic</t>
+  </si>
+  <si>
+    <t>Created scenes, nodes, scripts
+- created moveable buttons
+- started to implement recipes system
+- created cards and spawner</t>
+  </si>
+  <si>
+    <t>Fixed cooldown
+- Issues with certain weapons, e.g. singularity, fire staff</t>
   </si>
 </sst>
 </file>
@@ -249,7 +266,16 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="9">
+    <dxf>
+      <numFmt numFmtId="25" formatCode="hh:mm"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="25" formatCode="hh:mm"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="25" formatCode="hh:mm"/>
     </dxf>
@@ -282,15 +308,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G32" totalsRowShown="0">
-  <autoFilter ref="B6:G32" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G33" totalsRowShown="0">
+  <autoFilter ref="B6:G33" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{9EDA08BC-FC93-4374-BA7A-6AB42BF27608}" name="Date"/>
-    <tableColumn id="2" xr3:uid="{E52E82DE-B123-4B3E-8A7E-4FB2C6CEEE64}" name="Start" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{E52E82DE-B123-4B3E-8A7E-4FB2C6CEEE64}" name="Start" dataDxfId="8"/>
     <tableColumn id="3" xr3:uid="{385CF12C-F475-4237-A1B1-BA2B136D502D}" name="Finish"/>
     <tableColumn id="4" xr3:uid="{A53CF1BF-F8B6-4BD3-8E81-2C1B7E645EAD}" name="Task"/>
-    <tableColumn id="5" xr3:uid="{82A06DB5-D5A5-417C-9A3D-8CC5431A3DD7}" name="Details" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{6B5828D5-4B73-426F-9AEB-9B2280524C8F}" name="Time" dataDxfId="3">
+    <tableColumn id="5" xr3:uid="{82A06DB5-D5A5-417C-9A3D-8CC5431A3DD7}" name="Details" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{6B5828D5-4B73-426F-9AEB-9B2280524C8F}" name="Time" dataDxfId="6">
       <calculatedColumnFormula>IF(D7&lt;C7, D7+1, D7) - C7</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -299,6 +325,23 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{AE49BDCB-9AE2-4D8E-9526-2EE8E335347E}" name="Table24" displayName="Table24" ref="B6:G32" totalsRowShown="0">
+  <autoFilter ref="B6:G32" xr:uid="{AE49BDCB-9AE2-4D8E-9526-2EE8E335347E}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{FAD75835-A4A6-4918-9A7C-99AF5B35770D}" name="Date"/>
+    <tableColumn id="2" xr3:uid="{F0977FC6-F5CF-465A-9207-1F73F89AE501}" name="Start" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{AD0BF73D-5F1F-45CA-8916-5DFA51120605}" name="Finish"/>
+    <tableColumn id="4" xr3:uid="{4BFA8C06-23BA-461E-9D77-82786B1054D2}" name="Task"/>
+    <tableColumn id="5" xr3:uid="{6A295F47-2BD5-4F2C-9493-8C28EB221635}" name="Details" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{59C01672-DED4-421F-882C-FE79042D7229}" name="Time" dataDxfId="3">
+      <calculatedColumnFormula>IF(D7&lt;C7, D7+1, D7) - C7</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight18" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7A4A6574-3FF0-4809-85FD-1DDCB83EA4DD}" name="Table22" displayName="Table22" ref="A6:F11" totalsRowShown="0">
   <autoFilter ref="A6:F11" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
   <tableColumns count="6">
@@ -632,6 +675,591 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F0887D6-8664-4804-98D8-EE817E3A6A1B}">
+  <dimension ref="A1:I33"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="10.42578125" customWidth="1"/>
+    <col min="5" max="5" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="47.42578125" style="3" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" s="4" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="F1" s="5"/>
+    </row>
+    <row r="2" spans="1:9" s="4" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
+      <c r="A2" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="5"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="7">
+        <f>SUM(G7:G41)</f>
+        <v>3.067361111111111</v>
+      </c>
+      <c r="I4" s="2"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I5" s="2"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" t="s">
+        <v>4</v>
+      </c>
+      <c r="E6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G6" t="s">
+        <v>12</v>
+      </c>
+      <c r="I6" s="2"/>
+    </row>
+    <row r="7" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="B7" s="1">
+        <v>45738</v>
+      </c>
+      <c r="C7" s="2">
+        <v>0.625</v>
+      </c>
+      <c r="D7" s="2">
+        <v>0.77430555555555558</v>
+      </c>
+      <c r="E7" t="s">
+        <v>1</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="G7" s="2">
+        <f t="shared" ref="G7:G11" si="0">IF(D7&lt;C7, D7+1, D7) - C7</f>
+        <v>0.14930555555555558</v>
+      </c>
+      <c r="I7" s="2"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C8" s="2">
+        <v>0.87013888888888891</v>
+      </c>
+      <c r="D8" s="2">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="G8" s="2">
+        <f t="shared" si="0"/>
+        <v>0.17152777777777783</v>
+      </c>
+      <c r="I8" s="2"/>
+    </row>
+    <row r="9" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="B9" s="1">
+        <v>45739</v>
+      </c>
+      <c r="C9" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="D9" s="2">
+        <v>0.5625</v>
+      </c>
+      <c r="E9" t="s">
+        <v>1</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G9" s="2">
+        <f t="shared" si="0"/>
+        <v>6.25E-2</v>
+      </c>
+      <c r="I9" s="2"/>
+    </row>
+    <row r="10" spans="1:9" ht="105" x14ac:dyDescent="0.25">
+      <c r="C10" s="2">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="D10" s="2">
+        <v>0.88472222222222219</v>
+      </c>
+      <c r="E10" t="s">
+        <v>1</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="G10" s="2">
+        <f t="shared" si="0"/>
+        <v>9.3055555555555558E-2</v>
+      </c>
+      <c r="I10" s="2"/>
+    </row>
+    <row r="11" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="C11" s="2">
+        <v>0.97430555555555554</v>
+      </c>
+      <c r="D11" s="2">
+        <v>7.1527777777777773E-2</v>
+      </c>
+      <c r="E11" t="s">
+        <v>1</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G11" s="2">
+        <f t="shared" si="0"/>
+        <v>9.7222222222222321E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="B12" s="1">
+        <v>45740</v>
+      </c>
+      <c r="C12" s="2">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="D12" s="2">
+        <v>0.6875</v>
+      </c>
+      <c r="E12" t="s">
+        <v>1</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G12" s="2">
+        <f>IF(D12&lt;C12, D12+1, D12) - C12</f>
+        <v>0.14583333333333337</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="C13" s="2">
+        <v>0.98611111111111116</v>
+      </c>
+      <c r="D13" s="2">
+        <v>6.25E-2</v>
+      </c>
+      <c r="E13" t="s">
+        <v>1</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G13" s="2">
+        <f>IF(D13&lt;C13, D13+1, D13) - C13</f>
+        <v>7.638888888888884E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+      <c r="B14" s="1">
+        <v>45741</v>
+      </c>
+      <c r="C14" s="2">
+        <v>0.63888888888888884</v>
+      </c>
+      <c r="D14" s="2">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="E14" t="s">
+        <v>1</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G14" s="2">
+        <f>IF(D14&lt;C14, D14+1, D14) - C14</f>
+        <v>0.15277777777777779</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="C15" s="2">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="D15" s="2">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="E15" t="s">
+        <v>1</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="G15" s="2">
+        <f>IF(D15&lt;C15, D15+1, D15) - C15</f>
+        <v>8.3333333333333259E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="135" x14ac:dyDescent="0.25">
+      <c r="B16" s="1">
+        <v>45742</v>
+      </c>
+      <c r="C16" s="2">
+        <v>0.6875</v>
+      </c>
+      <c r="D16" s="2">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="E16" t="s">
+        <v>1</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G16" s="2">
+        <f>IF(D16&lt;C16, D16+1, D16) - C16</f>
+        <v>0.10416666666666663</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B17" s="1">
+        <v>45744</v>
+      </c>
+      <c r="C17" s="2">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="D17" s="2">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="E17" t="s">
+        <v>1</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G17" s="2">
+        <f t="shared" ref="G17:G20" si="1">IF(D17&lt;C17, D17+1, D17) - C17</f>
+        <v>0.25000000000000011</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B18" s="1">
+        <v>45745</v>
+      </c>
+      <c r="C18" s="2">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="D18" s="2">
+        <v>0.52083333333333337</v>
+      </c>
+      <c r="E18" t="s">
+        <v>1</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G18" s="2">
+        <f t="shared" si="1"/>
+        <v>6.2500000000000056E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="B19" s="1"/>
+      <c r="C19" s="2">
+        <v>0.625</v>
+      </c>
+      <c r="D19" s="2">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="E19" t="s">
+        <v>1</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="G19" s="2">
+        <f t="shared" si="1"/>
+        <v>0.16666666666666663</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B20" s="1"/>
+      <c r="C20" s="2">
+        <v>0.875</v>
+      </c>
+      <c r="D20" s="2">
+        <v>0.4375</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G20" s="2">
+        <f t="shared" si="1"/>
+        <v>0.5625</v>
+      </c>
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C21" s="2">
+        <v>0.98958333333333337</v>
+      </c>
+      <c r="D21" s="2">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G21" s="2">
+        <f t="shared" ref="G21:G27" si="2">IF(D21&lt;C21, D21+1, D21) - C21</f>
+        <v>5.208333333333337E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="2:7" ht="75" x14ac:dyDescent="0.25">
+      <c r="B22" s="1">
+        <v>45746</v>
+      </c>
+      <c r="C22" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="D22" s="2">
+        <v>0.61388888888888893</v>
+      </c>
+      <c r="E22" t="s">
+        <v>1</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G22" s="2">
+        <f t="shared" si="2"/>
+        <v>0.11388888888888893</v>
+      </c>
+    </row>
+    <row r="23" spans="2:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="C23" s="2">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="D23" s="2">
+        <v>0.85763888888888884</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G23" s="2">
+        <f t="shared" si="2"/>
+        <v>6.597222222222221E-2</v>
+      </c>
+    </row>
+    <row r="24" spans="2:7" ht="75" x14ac:dyDescent="0.25">
+      <c r="B24" s="1">
+        <v>45747</v>
+      </c>
+      <c r="C24" s="2">
+        <v>0.57291666666666663</v>
+      </c>
+      <c r="D24" s="2">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="E24" t="s">
+        <v>1</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="G24" s="2">
+        <f t="shared" si="2"/>
+        <v>9.375E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="2:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="C25" s="2">
+        <v>0.75902777777777775</v>
+      </c>
+      <c r="D25" s="2">
+        <v>0.79027777777777775</v>
+      </c>
+      <c r="E25" t="s">
+        <v>1</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G25" s="2">
+        <f t="shared" si="2"/>
+        <v>3.125E-2</v>
+      </c>
+    </row>
+    <row r="26" spans="2:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="C26" s="2">
+        <v>0.89583333333333337</v>
+      </c>
+      <c r="D26" s="2">
+        <v>0.98263888888888884</v>
+      </c>
+      <c r="E26" t="s">
+        <v>1</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G26" s="2">
+        <f t="shared" si="2"/>
+        <v>8.6805555555555469E-2</v>
+      </c>
+    </row>
+    <row r="27" spans="2:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="C27" s="2">
+        <v>3.472222222222222E-3</v>
+      </c>
+      <c r="D27" s="2">
+        <v>3.4722222222222224E-2</v>
+      </c>
+      <c r="E27" t="s">
+        <v>1</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G27" s="2">
+        <f t="shared" si="2"/>
+        <v>3.125E-2</v>
+      </c>
+    </row>
+    <row r="28" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B28" s="1">
+        <v>45749</v>
+      </c>
+      <c r="C28" s="2">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="D28" s="2">
+        <v>0.99305555555555558</v>
+      </c>
+      <c r="E28" t="s">
+        <v>1</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G28" s="2">
+        <f t="shared" ref="G28:G33" si="3">IF(D28&lt;C28, D28+1, D28) - C28</f>
+        <v>3.472222222222221E-2</v>
+      </c>
+    </row>
+    <row r="29" spans="2:7" ht="120" x14ac:dyDescent="0.25">
+      <c r="B29" s="1">
+        <v>45750</v>
+      </c>
+      <c r="C29" s="2">
+        <v>0.96180555555555558</v>
+      </c>
+      <c r="D29" s="2">
+        <v>3.7499999999999999E-2</v>
+      </c>
+      <c r="E29" t="s">
+        <v>1</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G29" s="2">
+        <f t="shared" si="3"/>
+        <v>7.5694444444444509E-2</v>
+      </c>
+    </row>
+    <row r="30" spans="2:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="B30" s="1">
+        <v>45751</v>
+      </c>
+      <c r="C30" s="2">
+        <v>0.6875</v>
+      </c>
+      <c r="D30" s="2">
+        <v>0.72569444444444442</v>
+      </c>
+      <c r="E30" t="s">
+        <v>1</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G30" s="2">
+        <f t="shared" si="3"/>
+        <v>3.819444444444442E-2</v>
+      </c>
+    </row>
+    <row r="31" spans="2:7" ht="75" x14ac:dyDescent="0.25">
+      <c r="C31" s="2">
+        <v>0.88124999999999998</v>
+      </c>
+      <c r="D31" s="2">
+        <v>0.91180555555555554</v>
+      </c>
+      <c r="E31" t="s">
+        <v>1</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G31" s="2">
+        <f t="shared" si="3"/>
+        <v>3.0555555555555558E-2</v>
+      </c>
+    </row>
+    <row r="32" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B32" s="1">
+        <v>45752</v>
+      </c>
+      <c r="C32" s="2">
+        <v>0.625</v>
+      </c>
+      <c r="D32" s="2">
+        <v>0.82291666666666663</v>
+      </c>
+      <c r="E32" t="s">
+        <v>1</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="G32" s="2">
+        <f t="shared" si="3"/>
+        <v>0.19791666666666663</v>
+      </c>
+    </row>
+    <row r="33" spans="2:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="B33" s="1">
+        <v>45753</v>
+      </c>
+      <c r="C33" s="2">
+        <v>0.6791666666666667</v>
+      </c>
+      <c r="D33" s="2">
+        <v>0.71666666666666667</v>
+      </c>
+      <c r="E33" t="s">
+        <v>1</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G33" s="2">
+        <f t="shared" si="3"/>
+        <v>3.7499999999999978E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8C0A223-2407-4505-BAD0-756DF8AFB831}">
   <dimension ref="A1:I32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -643,7 +1271,7 @@
   <sheetData>
     <row r="1" spans="1:9" s="4" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A1" s="4" t="s">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="F1" s="5"/>
     </row>
@@ -659,7 +1287,7 @@
       </c>
       <c r="D4" s="7">
         <f>SUM(G7:G41)</f>
-        <v>3.2833333333333332</v>
+        <v>0.10486111111111113</v>
       </c>
       <c r="I4" s="2"/>
     </row>
@@ -687,511 +1315,179 @@
       </c>
       <c r="I6" s="2"/>
     </row>
-    <row r="7" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="B7" s="1">
-        <v>45738</v>
+        <v>45753</v>
       </c>
       <c r="C7" s="2">
-        <v>0.625</v>
+        <v>0.45833333333333331</v>
       </c>
       <c r="D7" s="2">
-        <v>0.77430555555555558</v>
+        <v>0.56319444444444444</v>
       </c>
       <c r="E7" t="s">
-        <v>1</v>
+        <v>38</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>2</v>
+        <v>39</v>
       </c>
       <c r="G7" s="2">
-        <f t="shared" ref="G7:G11" si="0">IF(D7&lt;C7, D7+1, D7) - C7</f>
-        <v>0.14930555555555558</v>
+        <f t="shared" ref="G7" si="0">IF(D7&lt;C7, D7+1, D7) - C7</f>
+        <v>0.10486111111111113</v>
       </c>
       <c r="I7" s="2"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="C8" s="2">
-        <v>0.87013888888888891</v>
-      </c>
-      <c r="D8" s="2">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="G8" s="2">
-        <f t="shared" si="0"/>
-        <v>0.17152777777777783</v>
-      </c>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="G8" s="2"/>
       <c r="I8" s="2"/>
     </row>
-    <row r="9" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="B9" s="1">
-        <v>45739</v>
-      </c>
-      <c r="C9" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="D9" s="2">
-        <v>0.5625</v>
-      </c>
-      <c r="E9" t="s">
-        <v>1</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G9" s="2">
-        <f t="shared" si="0"/>
-        <v>6.25E-2</v>
-      </c>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B9" s="1"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="G9" s="2"/>
       <c r="I9" s="2"/>
     </row>
-    <row r="10" spans="1:9" ht="105" x14ac:dyDescent="0.25">
-      <c r="C10" s="2">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="D10" s="2">
-        <v>0.88472222222222219</v>
-      </c>
-      <c r="E10" t="s">
-        <v>1</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G10" s="2">
-        <f t="shared" si="0"/>
-        <v>9.3055555555555558E-2</v>
-      </c>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="G10" s="2"/>
       <c r="I10" s="2"/>
     </row>
-    <row r="11" spans="1:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="C11" s="2">
-        <v>0.97430555555555554</v>
-      </c>
-      <c r="D11" s="2">
-        <v>7.1527777777777773E-2</v>
-      </c>
-      <c r="E11" t="s">
-        <v>1</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G11" s="2">
-        <f t="shared" si="0"/>
-        <v>9.7222222222222321E-2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="B12" s="1">
-        <v>45740</v>
-      </c>
-      <c r="C12" s="2">
-        <v>0.54166666666666663</v>
-      </c>
-      <c r="D12" s="2">
-        <v>0.6875</v>
-      </c>
-      <c r="E12" t="s">
-        <v>1</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="G12" s="2">
-        <f>IF(D12&lt;C12, D12+1, D12) - C12</f>
-        <v>0.14583333333333337</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="60" x14ac:dyDescent="0.25">
-      <c r="C13" s="2">
-        <v>0.98611111111111116</v>
-      </c>
-      <c r="D13" s="2">
-        <v>6.25E-2</v>
-      </c>
-      <c r="E13" t="s">
-        <v>1</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G13" s="2">
-        <f>IF(D13&lt;C13, D13+1, D13) - C13</f>
-        <v>7.638888888888884E-2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" ht="75" x14ac:dyDescent="0.25">
-      <c r="B14" s="1">
-        <v>45741</v>
-      </c>
-      <c r="C14" s="2">
-        <v>0.63888888888888884</v>
-      </c>
-      <c r="D14" s="2">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="E14" t="s">
-        <v>1</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="G14" s="2">
-        <f>IF(D14&lt;C14, D14+1, D14) - C14</f>
-        <v>0.15277777777777779</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" ht="60" x14ac:dyDescent="0.25">
-      <c r="C15" s="2">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="D15" s="2">
-        <v>0.91666666666666663</v>
-      </c>
-      <c r="E15" t="s">
-        <v>1</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="G15" s="2">
-        <f>IF(D15&lt;C15, D15+1, D15) - C15</f>
-        <v>8.3333333333333259E-2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="135" x14ac:dyDescent="0.25">
-      <c r="B16" s="1">
-        <v>45742</v>
-      </c>
-      <c r="C16" s="2">
-        <v>0.6875</v>
-      </c>
-      <c r="D16" s="2">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="E16" t="s">
-        <v>1</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="G16" s="2">
-        <f>IF(D16&lt;C16, D16+1, D16) - C16</f>
-        <v>0.10416666666666663</v>
-      </c>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="G11" s="2"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B12" s="1"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="G12" s="2"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="G13" s="2"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B14" s="1"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="G14" s="2"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="G15" s="2"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B16" s="1"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="G16" s="2"/>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B17" s="1">
-        <v>45744</v>
-      </c>
-      <c r="C17" s="2">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="D17" s="2">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="E17" t="s">
-        <v>1</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="G17" s="2">
-        <f t="shared" ref="G17:G20" si="1">IF(D17&lt;C17, D17+1, D17) - C17</f>
-        <v>0.25000000000000011</v>
-      </c>
+      <c r="B17" s="1"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+      <c r="G17" s="2"/>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B18" s="1">
-        <v>45745</v>
-      </c>
-      <c r="C18" s="2">
-        <v>0.45833333333333331</v>
-      </c>
-      <c r="D18" s="2">
-        <v>0.52083333333333337</v>
-      </c>
-      <c r="E18" t="s">
-        <v>1</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="G18" s="2">
-        <f t="shared" si="1"/>
-        <v>6.2500000000000056E-2</v>
-      </c>
-    </row>
-    <row r="19" spans="2:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="B18" s="1"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="G18" s="2"/>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B19" s="1"/>
-      <c r="C19" s="2">
-        <v>0.625</v>
-      </c>
-      <c r="D19" s="2">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="E19" t="s">
-        <v>1</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="G19" s="2">
-        <f t="shared" si="1"/>
-        <v>0.16666666666666663</v>
-      </c>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="G19" s="2"/>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B20" s="1"/>
-      <c r="C20" s="2">
-        <v>0.875</v>
-      </c>
-      <c r="D20" s="2">
-        <v>0.4375</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G20" s="2">
-        <f t="shared" si="1"/>
-        <v>0.5625</v>
-      </c>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
+      <c r="G20" s="2"/>
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C21" s="2">
-        <v>0.98958333333333337</v>
-      </c>
-      <c r="D21" s="2">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G21" s="2">
-        <f t="shared" ref="G21:G27" si="2">IF(D21&lt;C21, D21+1, D21) - C21</f>
-        <v>5.208333333333337E-2</v>
-      </c>
-    </row>
-    <row r="22" spans="2:7" ht="75" x14ac:dyDescent="0.25">
-      <c r="B22" s="1">
-        <v>45746</v>
-      </c>
-      <c r="C22" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="D22" s="2">
-        <v>0.61388888888888893</v>
-      </c>
-      <c r="E22" t="s">
-        <v>1</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="G22" s="2">
-        <f t="shared" si="2"/>
-        <v>0.11388888888888893</v>
-      </c>
-    </row>
-    <row r="23" spans="2:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="C23" s="2">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="D23" s="2">
-        <v>0.85763888888888884</v>
-      </c>
-      <c r="F23" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="G23" s="2">
-        <f t="shared" si="2"/>
-        <v>6.597222222222221E-2</v>
-      </c>
-    </row>
-    <row r="24" spans="2:7" ht="75" x14ac:dyDescent="0.25">
-      <c r="B24" s="1">
-        <v>45747</v>
-      </c>
-      <c r="C24" s="2">
-        <v>0.57291666666666663</v>
-      </c>
-      <c r="D24" s="2">
-        <v>0.66666666666666663</v>
-      </c>
-      <c r="E24" t="s">
-        <v>1</v>
-      </c>
-      <c r="F24" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="G24" s="2">
-        <f t="shared" si="2"/>
-        <v>9.375E-2</v>
-      </c>
-    </row>
-    <row r="25" spans="2:7" ht="60" x14ac:dyDescent="0.25">
-      <c r="C25" s="2">
-        <v>0.75902777777777775</v>
-      </c>
-      <c r="D25" s="2">
-        <v>0.79027777777777775</v>
-      </c>
-      <c r="E25" t="s">
-        <v>1</v>
-      </c>
-      <c r="F25" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="G25" s="2">
-        <f t="shared" si="2"/>
-        <v>3.125E-2</v>
-      </c>
-    </row>
-    <row r="26" spans="2:7" ht="45" x14ac:dyDescent="0.25">
-      <c r="C26" s="2">
-        <v>0.89583333333333337</v>
-      </c>
-      <c r="D26" s="2">
-        <v>0.98263888888888884</v>
-      </c>
-      <c r="E26" t="s">
-        <v>1</v>
-      </c>
-      <c r="F26" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="G26" s="2">
-        <f t="shared" si="2"/>
-        <v>8.6805555555555469E-2</v>
-      </c>
-    </row>
-    <row r="27" spans="2:7" ht="45" x14ac:dyDescent="0.25">
-      <c r="C27" s="2">
-        <v>3.472222222222222E-3</v>
-      </c>
-      <c r="D27" s="2">
-        <v>3.4722222222222224E-2</v>
-      </c>
-      <c r="E27" t="s">
-        <v>1</v>
-      </c>
-      <c r="F27" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="G27" s="2">
-        <f t="shared" si="2"/>
-        <v>3.125E-2</v>
-      </c>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
+      <c r="G21" s="2"/>
+    </row>
+    <row r="22" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B22" s="1"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+      <c r="G22" s="2"/>
+    </row>
+    <row r="23" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
+      <c r="G23" s="2"/>
+    </row>
+    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B24" s="1"/>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+      <c r="G24" s="2"/>
+    </row>
+    <row r="25" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
+      <c r="G25" s="2"/>
+    </row>
+    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C26" s="2"/>
+      <c r="D26" s="2"/>
+      <c r="G26" s="2"/>
+    </row>
+    <row r="27" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
+      <c r="G27" s="2"/>
     </row>
     <row r="28" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B28" s="1">
-        <v>45749</v>
-      </c>
-      <c r="C28" s="2">
-        <v>0.95833333333333337</v>
-      </c>
-      <c r="D28" s="2">
-        <v>0.99305555555555558</v>
-      </c>
-      <c r="E28" t="s">
-        <v>1</v>
-      </c>
-      <c r="F28" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G28" s="2">
-        <f>IF(D28&lt;C28, D28+1, D28) - C28</f>
-        <v>3.472222222222221E-2</v>
-      </c>
-    </row>
-    <row r="29" spans="2:7" ht="120" x14ac:dyDescent="0.25">
-      <c r="B29" s="1">
-        <v>45750</v>
-      </c>
-      <c r="C29" s="2">
-        <v>0.96180555555555558</v>
-      </c>
-      <c r="D29" s="2">
-        <v>3.7499999999999999E-2</v>
-      </c>
-      <c r="E29" t="s">
-        <v>1</v>
-      </c>
-      <c r="F29" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="G29" s="2">
-        <f>IF(D29&lt;C29, D29+1, D29) - C29</f>
-        <v>7.5694444444444509E-2</v>
-      </c>
-    </row>
-    <row r="30" spans="2:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="B30" s="1">
-        <v>45751</v>
-      </c>
-      <c r="C30" s="2">
-        <v>0.6875</v>
-      </c>
-      <c r="D30" s="2">
-        <v>0.72569444444444442</v>
-      </c>
-      <c r="E30" t="s">
-        <v>1</v>
-      </c>
-      <c r="F30" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="G30" s="2">
-        <f>IF(D30&lt;C30, D30+1, D30) - C30</f>
-        <v>3.819444444444442E-2</v>
-      </c>
-    </row>
-    <row r="31" spans="2:7" ht="75" x14ac:dyDescent="0.25">
-      <c r="C31" s="2">
-        <v>0.88124999999999998</v>
-      </c>
-      <c r="D31" s="2">
-        <v>0.91180555555555554</v>
-      </c>
-      <c r="E31" t="s">
-        <v>1</v>
-      </c>
-      <c r="F31" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G31" s="2">
-        <f>IF(D31&lt;C31, D31+1, D31) - C31</f>
-        <v>3.0555555555555558E-2</v>
-      </c>
+      <c r="B28" s="1"/>
+      <c r="C28" s="2"/>
+      <c r="D28" s="2"/>
+      <c r="G28" s="2"/>
+    </row>
+    <row r="29" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B29" s="1"/>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
+      <c r="G29" s="2"/>
+    </row>
+    <row r="30" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B30" s="1"/>
+      <c r="C30" s="2"/>
+      <c r="D30" s="2"/>
+      <c r="G30" s="2"/>
+    </row>
+    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C31" s="2"/>
+      <c r="D31" s="2"/>
+      <c r="G31" s="2"/>
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B32" s="1">
-        <v>45752</v>
-      </c>
-      <c r="C32" s="2">
-        <v>0.54861111111111116</v>
-      </c>
-      <c r="E32" t="s">
-        <v>1</v>
-      </c>
-      <c r="F32" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G32" s="2">
-        <f>IF(D32&lt;C32, D32+1, D32) - C32</f>
-        <v>0.45138888888888884</v>
-      </c>
+      <c r="B32" s="1"/>
+      <c r="C32" s="2"/>
+      <c r="D32" s="2"/>
+      <c r="G32" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16EBAB43-9BF7-46C1-BE2D-33751923E718}">
   <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Fixed weapon cooldown issues
</commit_message>
<xml_diff>
--- a/SD_WorkLog.xlsx
+++ b/SD_WorkLog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adamj\Documents\Game Development\Godot\Smash Dungeon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78873092-0864-4483-A329-02093806C1A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BEAD224-1B87-4B31-BA0E-40DABC527693}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1560" yWindow="735" windowWidth="21600" windowHeight="11235" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="41">
   <si>
     <t>Smash Dungeon</t>
   </si>
@@ -308,8 +308,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G33" totalsRowShown="0">
-  <autoFilter ref="B6:G33" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G34" totalsRowShown="0">
+  <autoFilter ref="B6:G34" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{9EDA08BC-FC93-4374-BA7A-6AB42BF27608}" name="Date"/>
     <tableColumn id="2" xr3:uid="{E52E82DE-B123-4B3E-8A7E-4FB2C6CEEE64}" name="Start" dataDxfId="8"/>
@@ -675,7 +675,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F0887D6-8664-4804-98D8-EE817E3A6A1B}">
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -702,7 +702,7 @@
       </c>
       <c r="D4" s="7">
         <f>SUM(G7:G41)</f>
-        <v>3.067361111111111</v>
+        <v>3.1701388888888888</v>
       </c>
       <c r="I4" s="2"/>
     </row>
@@ -1247,6 +1247,18 @@
       <c r="G33" s="2">
         <f t="shared" si="3"/>
         <v>3.7499999999999978E-2</v>
+      </c>
+    </row>
+    <row r="34" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C34" s="2">
+        <v>0.89722222222222225</v>
+      </c>
+      <c r="E34" t="s">
+        <v>1</v>
+      </c>
+      <c r="G34" s="2">
+        <f>IF(D34&lt;C34, D34+1, D34) - C34</f>
+        <v>0.10277777777777775</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed cooldown meter, but needs to be created on start of arena
</commit_message>
<xml_diff>
--- a/SD_WorkLog.xlsx
+++ b/SD_WorkLog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adamj\Documents\Game Development\Godot\Smash Dungeon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BEAD224-1B87-4B31-BA0E-40DABC527693}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0C553CE-29F9-48BD-AA7F-24EB0444079B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1560" yWindow="735" windowWidth="21600" windowHeight="11235" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="45">
   <si>
     <t>Smash Dungeon</t>
   </si>
@@ -197,6 +197,21 @@
   <si>
     <t>Fixed cooldown
 - Issues with certain weapons, e.g. singularity, fire staff</t>
+  </si>
+  <si>
+    <t>Fixed bugs with cooldown/weapons
+- All weapons now working
+- Faster attacks
+- started trying to implement new cooldown UI</t>
+  </si>
+  <si>
+    <t>Need to get slower attacks trialed</t>
+  </si>
+  <si>
+    <t>change UI for cooldown</t>
+  </si>
+  <si>
+    <t>trial adding some new weapons?</t>
   </si>
 </sst>
 </file>
@@ -308,8 +323,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G34" totalsRowShown="0">
-  <autoFilter ref="B6:G34" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G37" totalsRowShown="0">
+  <autoFilter ref="B6:G37" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{9EDA08BC-FC93-4374-BA7A-6AB42BF27608}" name="Date"/>
     <tableColumn id="2" xr3:uid="{E52E82DE-B123-4B3E-8A7E-4FB2C6CEEE64}" name="Start" dataDxfId="8"/>
@@ -675,7 +690,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F0887D6-8664-4804-98D8-EE817E3A6A1B}">
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -702,7 +717,7 @@
       </c>
       <c r="D4" s="7">
         <f>SUM(G7:G41)</f>
-        <v>3.1701388888888888</v>
+        <v>3.1284722222222223</v>
       </c>
       <c r="I4" s="2"/>
     </row>
@@ -1249,16 +1264,52 @@
         <v>3.7499999999999978E-2</v>
       </c>
     </row>
-    <row r="34" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:7" ht="60" x14ac:dyDescent="0.25">
       <c r="C34" s="2">
         <v>0.89722222222222225</v>
       </c>
+      <c r="D34" s="2">
+        <v>0.95833333333333337</v>
+      </c>
       <c r="E34" t="s">
         <v>1</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>41</v>
       </c>
       <c r="G34" s="2">
         <f>IF(D34&lt;C34, D34+1, D34) - C34</f>
-        <v>0.10277777777777775</v>
+        <v>6.1111111111111116E-2</v>
+      </c>
+    </row>
+    <row r="35" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C35" s="2"/>
+      <c r="F35" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="G35" s="2">
+        <f>IF(D35&lt;C35, D35+1, D35) - C35</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C36" s="2"/>
+      <c r="F36" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="G36" s="2">
+        <f>IF(D36&lt;C36, D36+1, D36) - C36</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C37" s="2"/>
+      <c r="F37" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="G37" s="2">
+        <f>IF(D37&lt;C37, D37+1, D37) - C37</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added a friendly fire system
</commit_message>
<xml_diff>
--- a/SD_WorkLog.xlsx
+++ b/SD_WorkLog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adamj\Documents\Game Development\Godot\Smash Dungeon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0C553CE-29F9-48BD-AA7F-24EB0444079B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23FA38E0-245D-4B7B-B154-47B680BADBE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="735" windowWidth="21600" windowHeight="11235" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
+    <workbookView xWindow="2940" yWindow="2115" windowWidth="21600" windowHeight="11235" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
   </bookViews>
   <sheets>
     <sheet name="Smash Dungeon" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="52">
   <si>
     <t>Smash Dungeon</t>
   </si>
@@ -208,10 +208,32 @@
     <t>Need to get slower attacks trialed</t>
   </si>
   <si>
-    <t>change UI for cooldown</t>
-  </si>
-  <si>
     <t>trial adding some new weapons?</t>
+  </si>
+  <si>
+    <t>Changed UI for cooldown</t>
+  </si>
+  <si>
+    <t>Weapon System</t>
+  </si>
+  <si>
+    <t>Made some decisions on weapon progression in single player
+- persistent weapon with scaling, and weapon drops that carry over (timed or with limited projectiles)</t>
+  </si>
+  <si>
+    <t>Items/Tarot/Ritual</t>
+  </si>
+  <si>
+    <t>Conceptual work on how system might work</t>
+  </si>
+  <si>
+    <t>Added basic implemention of adding weapon sprites</t>
+  </si>
+  <si>
+    <t>Weapon Sprites</t>
+  </si>
+  <si>
+    <t>Adding Friendly Fire</t>
   </si>
 </sst>
 </file>
@@ -323,8 +345,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G37" totalsRowShown="0">
-  <autoFilter ref="B6:G37" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G44" totalsRowShown="0">
+  <autoFilter ref="B6:G44" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{9EDA08BC-FC93-4374-BA7A-6AB42BF27608}" name="Date"/>
     <tableColumn id="2" xr3:uid="{E52E82DE-B123-4B3E-8A7E-4FB2C6CEEE64}" name="Start" dataDxfId="8"/>
@@ -690,7 +712,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F0887D6-8664-4804-98D8-EE817E3A6A1B}">
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I44"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -716,8 +738,8 @@
         <v>11</v>
       </c>
       <c r="D4" s="7">
-        <f>SUM(G7:G41)</f>
-        <v>3.1284722222222223</v>
+        <f>SUM(G7:G45)</f>
+        <v>3.5784722222222221</v>
       </c>
       <c r="I4" s="2"/>
     </row>
@@ -1278,37 +1300,153 @@
         <v>41</v>
       </c>
       <c r="G34" s="2">
-        <f>IF(D34&lt;C34, D34+1, D34) - C34</f>
+        <f t="shared" ref="G34:G39" si="4">IF(D34&lt;C34, D34+1, D34) - C34</f>
         <v>6.1111111111111116E-2</v>
       </c>
     </row>
     <row r="35" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C35" s="2"/>
+      <c r="B35" s="1">
+        <v>45754</v>
+      </c>
+      <c r="C35" s="2">
+        <v>0.63541666666666663</v>
+      </c>
+      <c r="D35" s="2">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="E35" t="s">
+        <v>1</v>
+      </c>
       <c r="F35" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="G35" s="2">
+        <f t="shared" si="4"/>
+        <v>7.2916666666666741E-2</v>
+      </c>
+    </row>
+    <row r="36" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B36" s="1"/>
+      <c r="C36" s="2">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="D36" s="2">
+        <v>0.875</v>
+      </c>
+      <c r="E36" t="s">
+        <v>47</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="G36" s="2">
+        <f t="shared" si="4"/>
+        <v>0.16666666666666663</v>
+      </c>
+    </row>
+    <row r="37" spans="2:7" ht="75" x14ac:dyDescent="0.25">
+      <c r="C37" s="2">
+        <v>0.89097222222222228</v>
+      </c>
+      <c r="D37" s="2">
+        <v>0.93055555555555558</v>
+      </c>
+      <c r="E37" t="s">
+        <v>45</v>
+      </c>
+      <c r="F37" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="G37" s="2">
+        <f t="shared" si="4"/>
+        <v>3.9583333333333304E-2</v>
+      </c>
+    </row>
+    <row r="38" spans="2:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="C38" s="2">
+        <v>0.98611111111111116</v>
+      </c>
+      <c r="D38" s="2">
+        <v>6.9444444444444441E-3</v>
+      </c>
+      <c r="E38" t="s">
+        <v>50</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="G38" s="2">
+        <f t="shared" si="4"/>
+        <v>2.0833333333333259E-2</v>
+      </c>
+    </row>
+    <row r="39" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B39" s="1">
+        <v>45755</v>
+      </c>
+      <c r="C39" s="2">
+        <v>0.64583333333333337</v>
+      </c>
+      <c r="D39" s="2">
+        <v>0.69861111111111107</v>
+      </c>
+      <c r="E39" t="s">
+        <v>45</v>
+      </c>
+      <c r="F39" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="G39" s="2">
+        <f t="shared" si="4"/>
+        <v>5.2777777777777701E-2</v>
+      </c>
+    </row>
+    <row r="40" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B40" s="1"/>
+      <c r="C40" s="2">
+        <v>0.90277777777777779</v>
+      </c>
+      <c r="D40" s="2"/>
+      <c r="G40" s="2">
+        <f>IF(D40&lt;C40, D40+1, D40) - C40</f>
+        <v>9.722222222222221E-2</v>
+      </c>
+    </row>
+    <row r="41" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B41" s="1"/>
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
+      <c r="G41" s="2">
+        <f>IF(D41&lt;C41, D41+1, D41) - C41</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B42" s="1"/>
+      <c r="C42" s="2"/>
+      <c r="D42" s="2"/>
+      <c r="G42" s="2">
+        <f>IF(D42&lt;C42, D42+1, D42) - C42</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C43" s="2"/>
+      <c r="F43" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="G43" s="2">
+        <f t="shared" ref="G43:G44" si="5">IF(D43&lt;C43, D43+1, D43) - C43</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C44" s="2"/>
+      <c r="F44" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="G35" s="2">
-        <f>IF(D35&lt;C35, D35+1, D35) - C35</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C36" s="2"/>
-      <c r="F36" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="G36" s="2">
-        <f>IF(D36&lt;C36, D36+1, D36) - C36</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C37" s="2"/>
-      <c r="F37" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="G37" s="2">
-        <f>IF(D37&lt;C37, D37+1, D37) - C37</f>
+      <c r="G44" s="2">
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added friendly fire and now self-damage with 0.5 second delay when launched to prevent collision
</commit_message>
<xml_diff>
--- a/SD_WorkLog.xlsx
+++ b/SD_WorkLog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adamj\Documents\Game Development\Godot\Smash Dungeon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23FA38E0-245D-4B7B-B154-47B680BADBE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{043F9820-2F75-48C5-8F5C-1BD52AB13219}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2940" yWindow="2115" windowWidth="21600" windowHeight="11235" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
   </bookViews>
   <sheets>
     <sheet name="Smash Dungeon" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="54">
   <si>
     <t>Smash Dungeon</t>
   </si>
@@ -234,6 +234,12 @@
   </si>
   <si>
     <t>Adding Friendly Fire</t>
+  </si>
+  <si>
+    <t>Adding Friendly Fire and reordering CSV</t>
+  </si>
+  <si>
+    <t>Added Friendly fire - BUT THE WRONG MECHANIC!!!</t>
   </si>
 </sst>
 </file>
@@ -739,7 +745,7 @@
       </c>
       <c r="D4" s="7">
         <f>SUM(G7:G45)</f>
-        <v>3.5784722222222221</v>
+        <v>3.7680555555555548</v>
       </c>
       <c r="I4" s="2"/>
     </row>
@@ -1406,28 +1412,44 @@
       <c r="C40" s="2">
         <v>0.90277777777777779</v>
       </c>
-      <c r="D40" s="2"/>
+      <c r="D40" s="2">
+        <v>0.94444444444444442</v>
+      </c>
+      <c r="F40" s="3" t="s">
+        <v>52</v>
+      </c>
       <c r="G40" s="2">
         <f>IF(D40&lt;C40, D40+1, D40) - C40</f>
-        <v>9.722222222222221E-2</v>
+        <v>4.166666666666663E-2</v>
       </c>
     </row>
     <row r="41" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B41" s="1"/>
-      <c r="C41" s="2"/>
-      <c r="D41" s="2"/>
+      <c r="B41" s="1">
+        <v>45756</v>
+      </c>
+      <c r="C41" s="2">
+        <v>0.65972222222222221</v>
+      </c>
+      <c r="D41" s="2">
+        <v>0.75</v>
+      </c>
+      <c r="F41" s="3" t="s">
+        <v>53</v>
+      </c>
       <c r="G41" s="2">
         <f>IF(D41&lt;C41, D41+1, D41) - C41</f>
-        <v>0</v>
+        <v>9.027777777777779E-2</v>
       </c>
     </row>
     <row r="42" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B42" s="1"/>
-      <c r="C42" s="2"/>
+      <c r="C42" s="2">
+        <v>0.84513888888888888</v>
+      </c>
       <c r="D42" s="2"/>
       <c r="G42" s="2">
         <f>IF(D42&lt;C42, D42+1, D42) - C42</f>
-        <v>0</v>
+        <v>0.15486111111111112</v>
       </c>
     </row>
     <row r="43" spans="2:7" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
switching to json system
</commit_message>
<xml_diff>
--- a/SD_WorkLog.xlsx
+++ b/SD_WorkLog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adamj\Documents\Game Development\Godot\Smash Dungeon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{043F9820-2F75-48C5-8F5C-1BD52AB13219}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24B69246-6D31-4A24-A326-531A377A8009}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
+    <workbookView xWindow="2940" yWindow="2115" windowWidth="21600" windowHeight="11235" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
   </bookViews>
   <sheets>
     <sheet name="Smash Dungeon" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="56">
   <si>
     <t>Smash Dungeon</t>
   </si>
@@ -240,6 +240,12 @@
   </si>
   <si>
     <t>Added Friendly fire - BUT THE WRONG MECHANIC!!!</t>
+  </si>
+  <si>
+    <t>Added self-damage</t>
+  </si>
+  <si>
+    <t>Looking into JSON storage solution</t>
   </si>
 </sst>
 </file>
@@ -351,8 +357,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G44" totalsRowShown="0">
-  <autoFilter ref="B6:G44" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G46" totalsRowShown="0">
+  <autoFilter ref="B6:G46" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{9EDA08BC-FC93-4374-BA7A-6AB42BF27608}" name="Date"/>
     <tableColumn id="2" xr3:uid="{E52E82DE-B123-4B3E-8A7E-4FB2C6CEEE64}" name="Start" dataDxfId="8"/>
@@ -718,7 +724,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F0887D6-8664-4804-98D8-EE817E3A6A1B}">
-  <dimension ref="A1:I44"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -744,8 +750,8 @@
         <v>11</v>
       </c>
       <c r="D4" s="7">
-        <f>SUM(G7:G45)</f>
-        <v>3.7680555555555548</v>
+        <f>SUM(G7:G47)</f>
+        <v>4.0249999999999995</v>
       </c>
       <c r="I4" s="2"/>
     </row>
@@ -1446,28 +1452,58 @@
       <c r="C42" s="2">
         <v>0.84513888888888888</v>
       </c>
-      <c r="D42" s="2"/>
+      <c r="D42" s="2">
+        <v>0.9375</v>
+      </c>
+      <c r="F42" s="3" t="s">
+        <v>54</v>
+      </c>
       <c r="G42" s="2">
         <f>IF(D42&lt;C42, D42+1, D42) - C42</f>
-        <v>0.15486111111111112</v>
+        <v>9.2361111111111116E-2</v>
       </c>
     </row>
     <row r="43" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C43" s="2"/>
+      <c r="B43" s="1">
+        <v>45757</v>
+      </c>
+      <c r="C43" s="2">
+        <v>0.68055555555555558</v>
+      </c>
+      <c r="D43" s="2"/>
       <c r="F43" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="G43" s="2">
+        <f>IF(D43&lt;C43, D43+1, D43) - C43</f>
+        <v>0.31944444444444442</v>
+      </c>
+    </row>
+    <row r="44" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B44" s="1"/>
+      <c r="C44" s="2"/>
+      <c r="D44" s="2"/>
+      <c r="G44" s="2">
+        <f>IF(D44&lt;C44, D44+1, D44) - C44</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C45" s="2"/>
+      <c r="F45" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="G43" s="2">
-        <f t="shared" ref="G43:G44" si="5">IF(D43&lt;C43, D43+1, D43) - C43</f>
+      <c r="G45" s="2">
+        <f t="shared" ref="G45:G46" si="5">IF(D45&lt;C45, D45+1, D45) - C45</f>
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C44" s="2"/>
-      <c r="F44" s="3" t="s">
+    <row r="46" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C46" s="2"/>
+      <c r="F46" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="G44" s="2">
+      <c r="G46" s="2">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
started implementing new arena system
</commit_message>
<xml_diff>
--- a/SD_WorkLog.xlsx
+++ b/SD_WorkLog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adamj\Documents\Game Development\Godot\Smash Dungeon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A41044F3-C68E-4269-9428-95B23751C0DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8372AD3-B26D-4340-B87B-F937DF64035B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2940" yWindow="2115" windowWidth="21600" windowHeight="11235" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
   </bookViews>
   <sheets>
     <sheet name="Smash Dungeon" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="61">
   <si>
     <t>Smash Dungeon</t>
   </si>
@@ -255,6 +255,12 @@
   </si>
   <si>
     <t>Looking into fixing Singularity bomb</t>
+  </si>
+  <si>
+    <t>Level System</t>
+  </si>
+  <si>
+    <t>Starting to think about creating new levels</t>
   </si>
 </sst>
 </file>
@@ -341,10 +347,10 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -393,8 +399,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G47" totalsRowShown="0">
-  <autoFilter ref="B6:G47" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G48" totalsRowShown="0">
+  <autoFilter ref="B6:G48" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{9EDA08BC-FC93-4374-BA7A-6AB42BF27608}" name="Date"/>
     <tableColumn id="2" xr3:uid="{E52E82DE-B123-4B3E-8A7E-4FB2C6CEEE64}" name="Start" dataDxfId="8"/>
@@ -760,7 +766,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F0887D6-8664-4804-98D8-EE817E3A6A1B}">
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -786,8 +792,8 @@
         <v>11</v>
       </c>
       <c r="D4" s="7">
-        <f>SUM(G7:G47)</f>
-        <v>4.5180555555555557</v>
+        <f>SUM(G7:G48)</f>
+        <v>4.3618055555555557</v>
       </c>
       <c r="I4" s="2"/>
     </row>
@@ -1588,18 +1594,50 @@
       <c r="C47" s="2">
         <v>0.75</v>
       </c>
+      <c r="D47" s="2">
+        <v>0.8125</v>
+      </c>
+      <c r="E47" t="s">
+        <v>59</v>
+      </c>
+      <c r="F47" s="3" t="s">
+        <v>60</v>
+      </c>
       <c r="G47" s="2">
         <f>IF(D47&lt;C47, D47+1, D47) - C47</f>
-        <v>0.25</v>
+        <v>6.25E-2</v>
       </c>
     </row>
     <row r="48" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="F48" s="8" t="s">
+      <c r="C48" s="2">
+        <v>0.96875</v>
+      </c>
+      <c r="D48" s="2"/>
+      <c r="E48" t="s">
+        <v>59</v>
+      </c>
+      <c r="G48" s="2">
+        <f>IF(D48&lt;C48, D48+1, D48) - C48</f>
+        <v>3.125E-2</v>
+      </c>
+    </row>
+    <row r="49" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C49" s="2"/>
+      <c r="D49" s="2"/>
+      <c r="G49" s="2"/>
+    </row>
+    <row r="50" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C50" s="2"/>
+      <c r="D50" s="2"/>
+      <c r="G50" s="2"/>
+    </row>
+    <row r="51" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="F51" s="8" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="49" spans="6:6" x14ac:dyDescent="0.25">
-      <c r="F49" s="9" t="s">
+    <row r="52" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="F52" s="9" t="s">
         <v>42</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added new arena creator system
</commit_message>
<xml_diff>
--- a/SD_WorkLog.xlsx
+++ b/SD_WorkLog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adamj\Documents\Game Development\Godot\Smash Dungeon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8372AD3-B26D-4340-B87B-F937DF64035B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{980DF8E3-2FFE-4E87-BCFB-815898BDB5AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="63">
   <si>
     <t>Smash Dungeon</t>
   </si>
@@ -261,6 +261,20 @@
   </si>
   <si>
     <t>Starting to think about creating new levels</t>
+  </si>
+  <si>
+    <t>Implementing arena system
+- fixed connection between existing scenes to load arenas</t>
+  </si>
+  <si>
+    <t>Created new arena editor system:
+Successfully debugged and fixed the ArenaDatabase singleton loading issue (identified the has_singleton timing quirk and implemented the direct access workaround).
+Correctly integrated the GameManager, ArenaDatabase, and battle_arena scene flow for loading specific arena data.
+Set up and used the arena_capture_tool to save layout data, including dynamic spawn points via Marker2Ds.
+Successfully loaded and tested a second, different arena layout, proving the system's flexibility.
+Defined a solid schema for placeholder TileSet properties to enable rapid functional level design.
+Clarified how to handle backgrounds, parallax, decorations, and UI within this system.
+Discussed potential future AI approaches</t>
   </si>
 </sst>
 </file>
@@ -399,8 +413,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G48" totalsRowShown="0">
-  <autoFilter ref="B6:G48" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G50" totalsRowShown="0">
+  <autoFilter ref="B6:G50" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{9EDA08BC-FC93-4374-BA7A-6AB42BF27608}" name="Date"/>
     <tableColumn id="2" xr3:uid="{E52E82DE-B123-4B3E-8A7E-4FB2C6CEEE64}" name="Start" dataDxfId="8"/>
@@ -792,8 +806,8 @@
         <v>11</v>
       </c>
       <c r="D4" s="7">
-        <f>SUM(G7:G48)</f>
-        <v>4.3618055555555557</v>
+        <f>SUM(G7:G50)</f>
+        <v>4.7826388888888882</v>
       </c>
       <c r="I4" s="2"/>
     </row>
@@ -1621,22 +1635,51 @@
         <v>3.125E-2</v>
       </c>
     </row>
-    <row r="49" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C49" s="2"/>
-      <c r="D49" s="2"/>
-      <c r="G49" s="2"/>
-    </row>
-    <row r="50" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C50" s="2"/>
-      <c r="D50" s="2"/>
-      <c r="G50" s="2"/>
-    </row>
-    <row r="51" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="B49" s="1">
+        <v>45759</v>
+      </c>
+      <c r="C49" s="2">
+        <v>0.59097222222222223</v>
+      </c>
+      <c r="D49" s="2">
+        <v>0.71666666666666667</v>
+      </c>
+      <c r="E49" t="s">
+        <v>59</v>
+      </c>
+      <c r="F49" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="G49" s="2">
+        <f>IF(D49&lt;C49, D49+1, D49) - C49</f>
+        <v>0.12569444444444444</v>
+      </c>
+    </row>
+    <row r="50" spans="2:7" ht="360" x14ac:dyDescent="0.25">
+      <c r="C50" s="2">
+        <v>0.8</v>
+      </c>
+      <c r="D50" s="2">
+        <v>9.5138888888888884E-2</v>
+      </c>
+      <c r="E50" t="s">
+        <v>59</v>
+      </c>
+      <c r="F50" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="G50" s="2">
+        <f>IF(D50&lt;C50, D50+1, D50) - C50</f>
+        <v>0.29513888888888884</v>
+      </c>
+    </row>
+    <row r="51" spans="2:7" x14ac:dyDescent="0.25">
       <c r="F51" s="8" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="52" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:7" x14ac:dyDescent="0.25">
       <c r="F52" s="9" t="s">
         <v>42</v>
       </c>

</xml_diff>

<commit_message>
added new arena select screen and fixing attack styles after twin stick system
</commit_message>
<xml_diff>
--- a/SD_WorkLog.xlsx
+++ b/SD_WorkLog.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adamj\Documents\Game Development\Godot\Smash Dungeon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{980DF8E3-2FFE-4E87-BCFB-815898BDB5AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5F4BE9E-B4E4-4F28-855B-1676D2845E50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
   </bookViews>
   <sheets>
     <sheet name="Smash Dungeon" sheetId="1" r:id="rId1"/>
-    <sheet name="Card Combiner" sheetId="3" r:id="rId2"/>
-    <sheet name="Godot Learning" sheetId="2" r:id="rId3"/>
+    <sheet name="Name Ideas" sheetId="4" r:id="rId2"/>
+    <sheet name="Card Combiner" sheetId="3" r:id="rId3"/>
+    <sheet name="Godot Learning" sheetId="2" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="72">
   <si>
     <t>Smash Dungeon</t>
   </si>
@@ -275,6 +276,35 @@
 Defined a solid schema for placeholder TileSet properties to enable rapid functional level design.
 Clarified how to handle backgrounds, parallax, decorations, and UI within this system.
 Discussed potential future AI approaches</t>
+  </si>
+  <si>
+    <t>Added Twin-Stick control system 
+- Added bug, player character attacks in wrong direction</t>
+  </si>
+  <si>
+    <t>Marketing</t>
+  </si>
+  <si>
+    <t>Brainstorming names, etc</t>
+  </si>
+  <si>
+    <t>Name Ideas</t>
+  </si>
+  <si>
+    <t>Descendrum</t>
+  </si>
+  <si>
+    <t>Fixing wrong direction
+- attack styles were reversing direction being given by player and weapon base</t>
+  </si>
+  <si>
+    <t>Control</t>
+  </si>
+  <si>
+    <t>Bug Fix</t>
+  </si>
+  <si>
+    <t>Creating Arena Select Screen</t>
   </si>
 </sst>
 </file>
@@ -413,8 +443,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G50" totalsRowShown="0">
-  <autoFilter ref="B6:G50" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G55" totalsRowShown="0">
+  <autoFilter ref="B6:G55" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{9EDA08BC-FC93-4374-BA7A-6AB42BF27608}" name="Date"/>
     <tableColumn id="2" xr3:uid="{E52E82DE-B123-4B3E-8A7E-4FB2C6CEEE64}" name="Start" dataDxfId="8"/>
@@ -780,7 +810,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F0887D6-8664-4804-98D8-EE817E3A6A1B}">
-  <dimension ref="A1:I52"/>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -806,8 +836,8 @@
         <v>11</v>
       </c>
       <c r="D4" s="7">
-        <f>SUM(G7:G50)</f>
-        <v>4.7826388888888882</v>
+        <f>SUM(G7:G55)</f>
+        <v>5.1701388888888893</v>
       </c>
       <c r="I4" s="2"/>
     </row>
@@ -1656,7 +1686,7 @@
         <v>0.12569444444444444</v>
       </c>
     </row>
-    <row r="50" spans="2:7" ht="360" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:7" ht="372" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C50" s="2">
         <v>0.8</v>
       </c>
@@ -1674,13 +1704,110 @@
         <v>0.29513888888888884</v>
       </c>
     </row>
-    <row r="51" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="F51" s="8" t="s">
+    <row r="51" spans="2:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="B51" s="1">
+        <v>45760</v>
+      </c>
+      <c r="C51" s="2">
+        <v>0.55833333333333335</v>
+      </c>
+      <c r="D51" s="2">
+        <v>0.77083333333333337</v>
+      </c>
+      <c r="E51" t="s">
+        <v>69</v>
+      </c>
+      <c r="F51" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="G51" s="2">
+        <f>IF(D51&lt;C51, D51+1, D51) - C51</f>
+        <v>0.21250000000000002</v>
+      </c>
+    </row>
+    <row r="52" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C52" s="2">
+        <v>0.7993055555555556</v>
+      </c>
+      <c r="D52" s="2">
+        <v>0.85416666666666663</v>
+      </c>
+      <c r="E52" t="s">
+        <v>64</v>
+      </c>
+      <c r="F52" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G52" s="2">
+        <f>IF(D52&lt;C52, D52+1, D52) - C52</f>
+        <v>5.4861111111111027E-2</v>
+      </c>
+    </row>
+    <row r="53" spans="2:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="C53" s="2">
+        <v>0.84375</v>
+      </c>
+      <c r="D53" s="2">
+        <v>0.875</v>
+      </c>
+      <c r="E53" t="s">
+        <v>70</v>
+      </c>
+      <c r="F53" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="G53" s="2">
+        <f>IF(D53&lt;C53, D53+1, D53) - C53</f>
+        <v>3.125E-2</v>
+      </c>
+    </row>
+    <row r="54" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C54" s="2">
+        <v>0.875</v>
+      </c>
+      <c r="D54" s="2">
+        <v>0.92361111111111116</v>
+      </c>
+      <c r="F54" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="G54" s="2">
+        <f>IF(D54&lt;C54, D54+1, D54) - C54</f>
+        <v>4.861111111111116E-2</v>
+      </c>
+    </row>
+    <row r="55" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C55" s="2">
+        <v>0.95972222222222225</v>
+      </c>
+      <c r="D55" s="2"/>
+      <c r="G55" s="2">
+        <f>IF(D55&lt;C55, D55+1, D55) - C55</f>
+        <v>4.0277777777777746E-2</v>
+      </c>
+    </row>
+    <row r="56" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C56" s="2"/>
+      <c r="D56" s="2"/>
+      <c r="G56" s="2"/>
+    </row>
+    <row r="57" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C57" s="2"/>
+      <c r="D57" s="2"/>
+      <c r="G57" s="2"/>
+    </row>
+    <row r="58" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C58" s="2"/>
+      <c r="D58" s="2"/>
+      <c r="G58" s="2"/>
+    </row>
+    <row r="59" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="F59" s="8" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="52" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="F52" s="9" t="s">
+    <row r="60" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="F60" s="9" t="s">
         <v>42</v>
       </c>
     </row>
@@ -1694,6 +1821,26 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C79C026B-8D30-4100-A805-D11CB8F29CB9}">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8C0A223-2407-4505-BAD0-756DF8AFB831}">
   <dimension ref="A1:I32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1922,7 +2069,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16EBAB43-9BF7-46C1-BE2D-33751923E718}">
   <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
fixed attack style errors
</commit_message>
<xml_diff>
--- a/SD_WorkLog.xlsx
+++ b/SD_WorkLog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adamj\Documents\Game Development\Godot\Smash Dungeon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5F4BE9E-B4E4-4F28-855B-1676D2845E50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3307E71F-D078-4D41-969B-4E6DCFD5434D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="73">
   <si>
     <t>Smash Dungeon</t>
   </si>
@@ -256,9 +256,6 @@
   </si>
   <si>
     <t>Looking into fixing Singularity bomb</t>
-  </si>
-  <si>
-    <t>Level System</t>
   </si>
   <si>
     <t>Starting to think about creating new levels</t>
@@ -305,6 +302,12 @@
   </si>
   <si>
     <t>Creating Arena Select Screen</t>
+  </si>
+  <si>
+    <t>Arena System</t>
+  </si>
+  <si>
+    <t>Melee attack style crashing (something to do with attack_direction and timer? Need to check against other scripts and whole system</t>
   </si>
 </sst>
 </file>
@@ -837,7 +840,7 @@
       </c>
       <c r="D4" s="7">
         <f>SUM(G7:G55)</f>
-        <v>5.1701388888888893</v>
+        <v>5.1888888888888891</v>
       </c>
       <c r="I4" s="2"/>
     </row>
@@ -1642,13 +1645,13 @@
         <v>0.8125</v>
       </c>
       <c r="E47" t="s">
+        <v>71</v>
+      </c>
+      <c r="F47" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="F47" s="3" t="s">
-        <v>60</v>
-      </c>
       <c r="G47" s="2">
-        <f>IF(D47&lt;C47, D47+1, D47) - C47</f>
+        <f t="shared" ref="G47:G55" si="6">IF(D47&lt;C47, D47+1, D47) - C47</f>
         <v>6.25E-2</v>
       </c>
     </row>
@@ -1658,10 +1661,10 @@
       </c>
       <c r="D48" s="2"/>
       <c r="E48" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="G48" s="2">
-        <f>IF(D48&lt;C48, D48+1, D48) - C48</f>
+        <f t="shared" si="6"/>
         <v>3.125E-2</v>
       </c>
     </row>
@@ -1676,13 +1679,13 @@
         <v>0.71666666666666667</v>
       </c>
       <c r="E49" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G49" s="2">
-        <f>IF(D49&lt;C49, D49+1, D49) - C49</f>
+        <f t="shared" si="6"/>
         <v>0.12569444444444444</v>
       </c>
     </row>
@@ -1694,13 +1697,13 @@
         <v>9.5138888888888884E-2</v>
       </c>
       <c r="E50" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G50" s="2">
-        <f>IF(D50&lt;C50, D50+1, D50) - C50</f>
+        <f t="shared" si="6"/>
         <v>0.29513888888888884</v>
       </c>
     </row>
@@ -1715,13 +1718,13 @@
         <v>0.77083333333333337</v>
       </c>
       <c r="E51" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G51" s="2">
-        <f>IF(D51&lt;C51, D51+1, D51) - C51</f>
+        <f t="shared" si="6"/>
         <v>0.21250000000000002</v>
       </c>
     </row>
@@ -1733,13 +1736,13 @@
         <v>0.85416666666666663</v>
       </c>
       <c r="E52" t="s">
+        <v>63</v>
+      </c>
+      <c r="F52" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="F52" s="3" t="s">
-        <v>65</v>
-      </c>
       <c r="G52" s="2">
-        <f>IF(D52&lt;C52, D52+1, D52) - C52</f>
+        <f t="shared" si="6"/>
         <v>5.4861111111111027E-2</v>
       </c>
     </row>
@@ -1751,13 +1754,13 @@
         <v>0.875</v>
       </c>
       <c r="E53" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G53" s="2">
-        <f>IF(D53&lt;C53, D53+1, D53) - C53</f>
+        <f t="shared" si="6"/>
         <v>3.125E-2</v>
       </c>
     </row>
@@ -1768,22 +1771,33 @@
       <c r="D54" s="2">
         <v>0.92361111111111116</v>
       </c>
+      <c r="E54" t="s">
+        <v>71</v>
+      </c>
       <c r="F54" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G54" s="2">
-        <f>IF(D54&lt;C54, D54+1, D54) - C54</f>
+        <f t="shared" si="6"/>
         <v>4.861111111111116E-2</v>
       </c>
     </row>
-    <row r="55" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:7" ht="45" x14ac:dyDescent="0.25">
       <c r="C55" s="2">
         <v>0.95972222222222225</v>
       </c>
-      <c r="D55" s="2"/>
+      <c r="D55" s="2">
+        <v>1.8749999999999999E-2</v>
+      </c>
+      <c r="E55" t="s">
+        <v>69</v>
+      </c>
+      <c r="F55" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="G55" s="2">
-        <f>IF(D55&lt;C55, D55+1, D55) - C55</f>
-        <v>4.0277777777777746E-2</v>
+        <f t="shared" si="6"/>
+        <v>5.902777777777779E-2</v>
       </c>
     </row>
     <row r="56" spans="2:7" x14ac:dyDescent="0.25">
@@ -1827,12 +1841,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adding new enemy AI system
</commit_message>
<xml_diff>
--- a/SD_WorkLog.xlsx
+++ b/SD_WorkLog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adamj\Documents\Game Development\Godot\Smash Dungeon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3307E71F-D078-4D41-969B-4E6DCFD5434D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D3C0581-944B-44DD-A5C8-F00AF92AABE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="75">
   <si>
     <t>Smash Dungeon</t>
   </si>
@@ -308,6 +308,12 @@
   </si>
   <si>
     <t>Melee attack style crashing (something to do with attack_direction and timer? Need to check against other scripts and whole system</t>
+  </si>
+  <si>
+    <t>Rewrote attack style base and attack styles to centralize player direction, and included collision utils into attack styles</t>
+  </si>
+  <si>
+    <t>Enemy AI</t>
   </si>
 </sst>
 </file>
@@ -446,8 +452,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G55" totalsRowShown="0">
-  <autoFilter ref="B6:G55" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G57" totalsRowShown="0">
+  <autoFilter ref="B6:G57" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{9EDA08BC-FC93-4374-BA7A-6AB42BF27608}" name="Date"/>
     <tableColumn id="2" xr3:uid="{E52E82DE-B123-4B3E-8A7E-4FB2C6CEEE64}" name="Start" dataDxfId="8"/>
@@ -813,7 +819,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F0887D6-8664-4804-98D8-EE817E3A6A1B}">
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:I74"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -839,8 +845,8 @@
         <v>11</v>
       </c>
       <c r="D4" s="7">
-        <f>SUM(G7:G55)</f>
-        <v>5.1888888888888891</v>
+        <f>SUM(G7:G57)</f>
+        <v>5.5347222222222223</v>
       </c>
       <c r="I4" s="2"/>
     </row>
@@ -1800,28 +1806,136 @@
         <v>5.902777777777779E-2</v>
       </c>
     </row>
-    <row r="56" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C56" s="2"/>
-      <c r="D56" s="2"/>
-      <c r="G56" s="2"/>
+    <row r="56" spans="2:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="B56" s="1">
+        <v>45761</v>
+      </c>
+      <c r="C56" s="2">
+        <v>0.57638888888888884</v>
+      </c>
+      <c r="D56" s="2">
+        <v>0.61736111111111114</v>
+      </c>
+      <c r="E56" t="s">
+        <v>69</v>
+      </c>
+      <c r="F56" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="G56" s="2">
+        <f>IF(D56&lt;C56, D56+1, D56) - C56</f>
+        <v>4.0972222222222299E-2</v>
+      </c>
     </row>
     <row r="57" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C57" s="2"/>
+      <c r="B57" s="1"/>
+      <c r="C57" s="2">
+        <v>0.69513888888888886</v>
+      </c>
       <c r="D57" s="2"/>
-      <c r="G57" s="2"/>
+      <c r="E57" t="s">
+        <v>74</v>
+      </c>
+      <c r="G57" s="2">
+        <f>IF(D57&lt;C57, D57+1, D57) - C57</f>
+        <v>0.30486111111111114</v>
+      </c>
     </row>
     <row r="58" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B58" s="1"/>
       <c r="C58" s="2"/>
       <c r="D58" s="2"/>
       <c r="G58" s="2"/>
     </row>
     <row r="59" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="F59" s="8" t="s">
+      <c r="B59" s="1"/>
+      <c r="C59" s="2"/>
+      <c r="D59" s="2"/>
+      <c r="G59" s="2"/>
+    </row>
+    <row r="60" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B60" s="1"/>
+      <c r="C60" s="2"/>
+      <c r="D60" s="2"/>
+      <c r="G60" s="2"/>
+    </row>
+    <row r="61" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B61" s="1"/>
+      <c r="C61" s="2"/>
+      <c r="D61" s="2"/>
+      <c r="G61" s="2"/>
+    </row>
+    <row r="62" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B62" s="1"/>
+      <c r="C62" s="2"/>
+      <c r="D62" s="2"/>
+      <c r="G62" s="2"/>
+    </row>
+    <row r="63" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B63" s="1"/>
+      <c r="C63" s="2"/>
+      <c r="D63" s="2"/>
+      <c r="G63" s="2"/>
+    </row>
+    <row r="64" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B64" s="1"/>
+      <c r="C64" s="2"/>
+      <c r="D64" s="2"/>
+      <c r="G64" s="2"/>
+    </row>
+    <row r="65" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B65" s="1"/>
+      <c r="C65" s="2"/>
+      <c r="D65" s="2"/>
+      <c r="G65" s="2"/>
+    </row>
+    <row r="66" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B66" s="1"/>
+      <c r="C66" s="2"/>
+      <c r="D66" s="2"/>
+      <c r="G66" s="2"/>
+    </row>
+    <row r="67" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B67" s="1"/>
+      <c r="C67" s="2"/>
+      <c r="D67" s="2"/>
+      <c r="G67" s="2"/>
+    </row>
+    <row r="68" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B68" s="1"/>
+      <c r="C68" s="2"/>
+      <c r="D68" s="2"/>
+      <c r="G68" s="2"/>
+    </row>
+    <row r="69" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B69" s="1"/>
+      <c r="C69" s="2"/>
+      <c r="D69" s="2"/>
+      <c r="G69" s="2"/>
+    </row>
+    <row r="70" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B70" s="1"/>
+      <c r="C70" s="2"/>
+      <c r="D70" s="2"/>
+      <c r="G70" s="2"/>
+    </row>
+    <row r="71" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C71" s="2"/>
+      <c r="D71" s="2"/>
+      <c r="G71" s="2"/>
+    </row>
+    <row r="72" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C72" s="2"/>
+      <c r="D72" s="2"/>
+      <c r="G72" s="2"/>
+    </row>
+    <row r="73" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="F73" s="8" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="60" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="F60" s="9" t="s">
+    <row r="74" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="F74" s="9" t="s">
         <v>42</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added some new procedural enemies to test
</commit_message>
<xml_diff>
--- a/SD_WorkLog.xlsx
+++ b/SD_WorkLog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adamj\Documents\Game Development\Godot\Smash Dungeon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D3C0581-944B-44DD-A5C8-F00AF92AABE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A946C1B4-0E02-47D3-AAA8-1025F4091EA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11235" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
   </bookViews>
   <sheets>
     <sheet name="Smash Dungeon" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="78">
   <si>
     <t>Smash Dungeon</t>
   </si>
@@ -313,7 +313,24 @@
     <t>Rewrote attack style base and attack styles to centralize player direction, and included collision utils into attack styles</t>
   </si>
   <si>
-    <t>Enemy AI</t>
+    <t>Enemy System</t>
+  </si>
+  <si>
+    <t>Created new Enemy System:
+- Enemy Manager
+- Enemy config
+- Basic Enemy
+- Slime (attempt to create procedural slime enemy)
+- Slime spit</t>
+  </si>
+  <si>
+    <t>Added slithering limb</t>
+  </si>
+  <si>
+    <t>Added more basic enemies:
+- bouncer
+- jumper
+- turret</t>
   </si>
 </sst>
 </file>
@@ -452,8 +469,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G57" totalsRowShown="0">
-  <autoFilter ref="B6:G57" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G60" totalsRowShown="0">
+  <autoFilter ref="B6:G60" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{9EDA08BC-FC93-4374-BA7A-6AB42BF27608}" name="Date"/>
     <tableColumn id="2" xr3:uid="{E52E82DE-B123-4B3E-8A7E-4FB2C6CEEE64}" name="Start" dataDxfId="8"/>
@@ -845,8 +862,8 @@
         <v>11</v>
       </c>
       <c r="D4" s="7">
-        <f>SUM(G7:G57)</f>
-        <v>5.5347222222222223</v>
+        <f>SUM(G7:G60)</f>
+        <v>6.1958333333333337</v>
       </c>
       <c r="I4" s="2"/>
     </row>
@@ -1827,37 +1844,75 @@
         <v>4.0972222222222299E-2</v>
       </c>
     </row>
-    <row r="57" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:7" ht="90" x14ac:dyDescent="0.25">
       <c r="B57" s="1"/>
       <c r="C57" s="2">
         <v>0.69513888888888886</v>
       </c>
-      <c r="D57" s="2"/>
+      <c r="D57" s="2">
+        <v>0.92638888888888893</v>
+      </c>
       <c r="E57" t="s">
         <v>74</v>
       </c>
+      <c r="F57" s="3" t="s">
+        <v>75</v>
+      </c>
       <c r="G57" s="2">
         <f>IF(D57&lt;C57, D57+1, D57) - C57</f>
-        <v>0.30486111111111114</v>
+        <v>0.23125000000000007</v>
       </c>
     </row>
     <row r="58" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B58" s="1"/>
-      <c r="C58" s="2"/>
-      <c r="D58" s="2"/>
-      <c r="G58" s="2"/>
+      <c r="B58" s="1">
+        <v>45762</v>
+      </c>
+      <c r="C58" s="2">
+        <v>1.0416666666666666E-2</v>
+      </c>
+      <c r="D58" s="2">
+        <v>5.7638888888888892E-2</v>
+      </c>
+      <c r="E58" t="s">
+        <v>74</v>
+      </c>
+      <c r="G58" s="2">
+        <f>IF(D58&lt;C58, D58+1, D58) - C58</f>
+        <v>4.7222222222222228E-2</v>
+      </c>
     </row>
     <row r="59" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B59" s="1"/>
-      <c r="C59" s="2"/>
-      <c r="D59" s="2"/>
-      <c r="G59" s="2"/>
-    </row>
-    <row r="60" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C59" s="2">
+        <v>0.6875</v>
+      </c>
+      <c r="D59" s="2">
+        <v>0.8125</v>
+      </c>
+      <c r="E59" t="s">
+        <v>74</v>
+      </c>
+      <c r="F59" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="G59" s="2">
+        <f>IF(D59&lt;C59, D59+1, D59) - C59</f>
+        <v>0.125</v>
+      </c>
+    </row>
+    <row r="60" spans="2:7" ht="60" x14ac:dyDescent="0.25">
       <c r="B60" s="1"/>
-      <c r="C60" s="2"/>
+      <c r="C60" s="2">
+        <v>0.4375</v>
+      </c>
       <c r="D60" s="2"/>
-      <c r="G60" s="2"/>
+      <c r="F60" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="G60" s="2">
+        <f>IF(D60&lt;C60, D60+1, D60) - C60</f>
+        <v>0.5625</v>
+      </c>
     </row>
     <row r="61" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B61" s="1"/>

</xml_diff>

<commit_message>
adding dynamic navigation for enemies
</commit_message>
<xml_diff>
--- a/SD_WorkLog.xlsx
+++ b/SD_WorkLog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adamj\Documents\Game Development\Godot\Smash Dungeon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A946C1B4-0E02-47D3-AAA8-1025F4091EA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C5158B3-95D8-41D3-A759-33D4525E7469}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11235" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="86">
   <si>
     <t>Smash Dungeon</t>
   </si>
@@ -330,7 +330,34 @@
     <t>Added more basic enemies:
 - bouncer
 - jumper
-- turret</t>
+- turret
+- procedural spider
+- procedural spider 3d
+- carrion beast</t>
+  </si>
+  <si>
+    <t>Trying to fix hitboxes for pull blade and blast hammer</t>
+  </si>
+  <si>
+    <t>Bug fix</t>
+  </si>
+  <si>
+    <t>Fixed hitboxes for pull blade and blast hammer</t>
+  </si>
+  <si>
+    <t>Centralised collisions for weapons</t>
+  </si>
+  <si>
+    <t>Creating a new enemy</t>
+  </si>
+  <si>
+    <t>Descendom</t>
+  </si>
+  <si>
+    <t>Fixing projectile collisions</t>
+  </si>
+  <si>
+    <t>Fixing dagger</t>
   </si>
 </sst>
 </file>
@@ -469,8 +496,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G60" totalsRowShown="0">
-  <autoFilter ref="B6:G60" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G66" totalsRowShown="0">
+  <autoFilter ref="B6:G66" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{9EDA08BC-FC93-4374-BA7A-6AB42BF27608}" name="Date"/>
     <tableColumn id="2" xr3:uid="{E52E82DE-B123-4B3E-8A7E-4FB2C6CEEE64}" name="Start" dataDxfId="8"/>
@@ -862,8 +889,8 @@
         <v>11</v>
       </c>
       <c r="D4" s="7">
-        <f>SUM(G7:G60)</f>
-        <v>6.1958333333333337</v>
+        <f>SUM(G7:G66)</f>
+        <v>6.5666666666666664</v>
       </c>
       <c r="I4" s="2"/>
     </row>
@@ -1840,7 +1867,7 @@
         <v>73</v>
       </c>
       <c r="G56" s="2">
-        <f>IF(D56&lt;C56, D56+1, D56) - C56</f>
+        <f t="shared" ref="G56:G65" si="7">IF(D56&lt;C56, D56+1, D56) - C56</f>
         <v>4.0972222222222299E-2</v>
       </c>
     </row>
@@ -1859,7 +1886,7 @@
         <v>75</v>
       </c>
       <c r="G57" s="2">
-        <f>IF(D57&lt;C57, D57+1, D57) - C57</f>
+        <f t="shared" si="7"/>
         <v>0.23125000000000007</v>
       </c>
     </row>
@@ -1877,7 +1904,7 @@
         <v>74</v>
       </c>
       <c r="G58" s="2">
-        <f>IF(D58&lt;C58, D58+1, D58) - C58</f>
+        <f t="shared" si="7"/>
         <v>4.7222222222222228E-2</v>
       </c>
     </row>
@@ -1896,59 +1923,128 @@
         <v>76</v>
       </c>
       <c r="G59" s="2">
-        <f>IF(D59&lt;C59, D59+1, D59) - C59</f>
+        <f t="shared" si="7"/>
         <v>0.125</v>
       </c>
     </row>
-    <row r="60" spans="2:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:7" ht="105" x14ac:dyDescent="0.25">
       <c r="B60" s="1"/>
       <c r="C60" s="2">
-        <v>0.4375</v>
-      </c>
-      <c r="D60" s="2"/>
+        <v>0.9375</v>
+      </c>
+      <c r="D60" s="2">
+        <v>7.2916666666666671E-2</v>
+      </c>
       <c r="F60" s="3" t="s">
         <v>77</v>
       </c>
       <c r="G60" s="2">
-        <f>IF(D60&lt;C60, D60+1, D60) - C60</f>
-        <v>0.5625</v>
-      </c>
-    </row>
-    <row r="61" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B61" s="1"/>
-      <c r="C61" s="2"/>
-      <c r="D61" s="2"/>
-      <c r="G61" s="2"/>
+        <f t="shared" si="7"/>
+        <v>0.13541666666666674</v>
+      </c>
+    </row>
+    <row r="61" spans="2:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="B61" s="1">
+        <v>45764</v>
+      </c>
+      <c r="C61" s="2">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="D61" s="2">
+        <v>1.6666666666666666E-2</v>
+      </c>
+      <c r="E61" t="s">
+        <v>69</v>
+      </c>
+      <c r="F61" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="G61" s="2">
+        <f t="shared" si="7"/>
+        <v>9.9999999999999978E-2</v>
+      </c>
     </row>
     <row r="62" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B62" s="1"/>
-      <c r="C62" s="2"/>
-      <c r="D62" s="2"/>
-      <c r="G62" s="2"/>
+      <c r="B62" s="1">
+        <v>45765</v>
+      </c>
+      <c r="C62" s="2">
+        <v>0.86805555555555558</v>
+      </c>
+      <c r="D62" s="2">
+        <v>1.0416666666666666E-2</v>
+      </c>
+      <c r="E62" t="s">
+        <v>79</v>
+      </c>
+      <c r="F62" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="G62" s="2">
+        <f t="shared" si="7"/>
+        <v>0.14236111111111116</v>
+      </c>
     </row>
     <row r="63" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B63" s="1"/>
       <c r="C63" s="2"/>
       <c r="D63" s="2"/>
-      <c r="G63" s="2"/>
+      <c r="E63" t="s">
+        <v>74</v>
+      </c>
+      <c r="F63" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="G63" s="2">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="64" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B64" s="1"/>
       <c r="C64" s="2"/>
       <c r="D64" s="2"/>
-      <c r="G64" s="2"/>
+      <c r="E64" t="s">
+        <v>45</v>
+      </c>
+      <c r="F64" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="G64" s="2">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="65" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B65" s="1"/>
-      <c r="C65" s="2"/>
+      <c r="B65" s="1">
+        <v>45766</v>
+      </c>
+      <c r="C65" s="2">
+        <v>0.44444444444444442</v>
+      </c>
       <c r="D65" s="2"/>
-      <c r="G65" s="2"/>
+      <c r="E65" t="s">
+        <v>45</v>
+      </c>
+      <c r="F65" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="G65" s="2">
+        <f t="shared" si="7"/>
+        <v>0.55555555555555558</v>
+      </c>
     </row>
     <row r="66" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B66" s="1"/>
       <c r="C66" s="2"/>
       <c r="D66" s="2"/>
-      <c r="G66" s="2"/>
+      <c r="F66" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="G66" s="2">
+        <f>IF(D66&lt;C66, D66+1, D66) - C66</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="67" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B67" s="1"/>
@@ -2005,7 +2101,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C79C026B-8D30-4100-A805-D11CB8F29CB9}">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -2016,6 +2112,11 @@
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>66</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added new enemy system and integrated with weapon system. Also started an arena creator
</commit_message>
<xml_diff>
--- a/SD_WorkLog.xlsx
+++ b/SD_WorkLog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adamj\Documents\Game Development\Godot\Smash Dungeon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C5158B3-95D8-41D3-A759-33D4525E7469}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E50B21B4-C8B9-4A91-BC12-E2A3F6363E3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11235" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="92">
   <si>
     <t>Smash Dungeon</t>
   </si>
@@ -354,10 +354,31 @@
     <t>Descendom</t>
   </si>
   <si>
-    <t>Fixing projectile collisions</t>
-  </si>
-  <si>
-    <t>Fixing dagger</t>
+    <t>Fixing projectile collisions
+- Fixing dagger</t>
+  </si>
+  <si>
+    <t>Creating enemy navigation system</t>
+  </si>
+  <si>
+    <t>Fixed enemy navigation</t>
+  </si>
+  <si>
+    <t>Began refactoring enemy system</t>
+  </si>
+  <si>
+    <t>Enemies</t>
+  </si>
+  <si>
+    <t>Finished first refactoring of enemy system</t>
+  </si>
+  <si>
+    <t>Added Fodder enemy
+- added zap fodder enemy
+- created centralised weapon system for enemies to prevent references spread out across enemy script</t>
+  </si>
+  <si>
+    <t>Adding weapon system to remaining enemies</t>
   </si>
 </sst>
 </file>
@@ -496,8 +517,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G66" totalsRowShown="0">
-  <autoFilter ref="B6:G66" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G71" totalsRowShown="0">
+  <autoFilter ref="B6:G71" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{9EDA08BC-FC93-4374-BA7A-6AB42BF27608}" name="Date"/>
     <tableColumn id="2" xr3:uid="{E52E82DE-B123-4B3E-8A7E-4FB2C6CEEE64}" name="Start" dataDxfId="8"/>
@@ -889,8 +910,8 @@
         <v>11</v>
       </c>
       <c r="D4" s="7">
-        <f>SUM(G7:G66)</f>
-        <v>6.5666666666666664</v>
+        <f>SUM(G7:G71)</f>
+        <v>7.3513888888888888</v>
       </c>
       <c r="I4" s="2"/>
     </row>
@@ -2015,14 +2036,16 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:7" ht="30" x14ac:dyDescent="0.25">
       <c r="B65" s="1">
         <v>45766</v>
       </c>
       <c r="C65" s="2">
         <v>0.44444444444444442</v>
       </c>
-      <c r="D65" s="2"/>
+      <c r="D65" s="2">
+        <v>0.60416666666666663</v>
+      </c>
       <c r="E65" t="s">
         <v>45</v>
       </c>
@@ -2031,49 +2054,121 @@
       </c>
       <c r="G65" s="2">
         <f t="shared" si="7"/>
-        <v>0.55555555555555558</v>
+        <v>0.15972222222222221</v>
       </c>
     </row>
     <row r="66" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B66" s="1"/>
-      <c r="C66" s="2"/>
-      <c r="D66" s="2"/>
+      <c r="C66" s="2">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="D66" s="2">
+        <v>0.80486111111111114</v>
+      </c>
+      <c r="E66" t="s">
+        <v>74</v>
+      </c>
       <c r="F66" s="3" t="s">
         <v>85</v>
       </c>
       <c r="G66" s="2">
         <f>IF(D66&lt;C66, D66+1, D66) - C66</f>
-        <v>0</v>
+        <v>0.13819444444444451</v>
       </c>
     </row>
     <row r="67" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B67" s="1"/>
-      <c r="C67" s="2"/>
-      <c r="D67" s="2"/>
-      <c r="G67" s="2"/>
+      <c r="C67" s="2">
+        <v>0.86805555555555558</v>
+      </c>
+      <c r="D67" s="2">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="F67" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="G67" s="2">
+        <f>IF(D67&lt;C67, D67+1, D67) - C67</f>
+        <v>4.8611111111111049E-2</v>
+      </c>
     </row>
     <row r="68" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B68" s="1"/>
-      <c r="C68" s="2"/>
-      <c r="D68" s="2"/>
-      <c r="G68" s="2"/>
+      <c r="C68" s="2">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="D68" s="2">
+        <v>6.9444444444444441E-3</v>
+      </c>
+      <c r="E68" t="s">
+        <v>74</v>
+      </c>
+      <c r="F68" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="G68" s="2">
+        <f>IF(D68&lt;C68, D68+1, D68) - C68</f>
+        <v>9.027777777777779E-2</v>
+      </c>
     </row>
     <row r="69" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B69" s="1"/>
-      <c r="C69" s="2"/>
-      <c r="D69" s="2"/>
-      <c r="G69" s="2"/>
-    </row>
-    <row r="70" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B69" s="1">
+        <v>45767</v>
+      </c>
+      <c r="C69" s="2">
+        <v>0.65972222222222221</v>
+      </c>
+      <c r="D69" s="2">
+        <v>0.74513888888888891</v>
+      </c>
+      <c r="E69" t="s">
+        <v>74</v>
+      </c>
+      <c r="F69" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="G69" s="2">
+        <f>IF(D69&lt;C69, D69+1, D69) - C69</f>
+        <v>8.5416666666666696E-2</v>
+      </c>
+    </row>
+    <row r="70" spans="2:7" ht="60" x14ac:dyDescent="0.25">
       <c r="B70" s="1"/>
-      <c r="C70" s="2"/>
-      <c r="D70" s="2"/>
-      <c r="G70" s="2"/>
+      <c r="C70" s="2">
+        <v>0.89652777777777781</v>
+      </c>
+      <c r="D70" s="2">
+        <v>0.12430555555555556</v>
+      </c>
+      <c r="E70" t="s">
+        <v>88</v>
+      </c>
+      <c r="F70" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="G70" s="2">
+        <f>IF(D70&lt;C70, D70+1, D70) - C70</f>
+        <v>0.22777777777777763</v>
+      </c>
     </row>
     <row r="71" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C71" s="2"/>
+      <c r="B71" s="1">
+        <v>45768</v>
+      </c>
+      <c r="C71" s="2">
+        <v>0.40972222222222221</v>
+      </c>
       <c r="D71" s="2"/>
-      <c r="G71" s="2"/>
+      <c r="E71" t="s">
+        <v>88</v>
+      </c>
+      <c r="F71" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="G71" s="2">
+        <f>IF(D71&lt;C71, D71+1, D71) - C71</f>
+        <v>0.59027777777777779</v>
+      </c>
     </row>
     <row r="72" spans="2:7" x14ac:dyDescent="0.25">
       <c r="C72" s="2"/>

</xml_diff>

<commit_message>
Failed clinger experiment with component system
</commit_message>
<xml_diff>
--- a/SD_WorkLog.xlsx
+++ b/SD_WorkLog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adamj\Documents\Game Development\Godot\Smash Dungeon\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E50B21B4-C8B9-4A91-BC12-E2A3F6363E3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{613D1195-1830-4B76-A1CD-FA9F9BFDA16D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11235" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
+    <workbookView xWindow="5295" yWindow="2445" windowWidth="21600" windowHeight="11235" xr2:uid="{F19D98A7-6420-4EF7-85AF-F6CF1D239D63}"/>
   </bookViews>
   <sheets>
     <sheet name="Smash Dungeon" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="97">
   <si>
     <t>Smash Dungeon</t>
   </si>
@@ -379,6 +379,21 @@
   </si>
   <si>
     <t>Adding weapon system to remaining enemies</t>
+  </si>
+  <si>
+    <t>Added arena procedural generation</t>
+  </si>
+  <si>
+    <t>Adding new component enemy</t>
+  </si>
+  <si>
+    <t>Components and component configs</t>
+  </si>
+  <si>
+    <t>Trying to get surface clinger to work</t>
+  </si>
+  <si>
+    <t>Surface Clinger</t>
   </si>
 </sst>
 </file>
@@ -517,8 +532,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G71" totalsRowShown="0">
-  <autoFilter ref="B6:G71" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}" name="Table2" displayName="Table2" ref="B6:G78" totalsRowShown="0">
+  <autoFilter ref="B6:G78" xr:uid="{B1FBB0C8-47CA-4FE8-A951-187DAAFDBA3A}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{9EDA08BC-FC93-4374-BA7A-6AB42BF27608}" name="Date"/>
     <tableColumn id="2" xr3:uid="{E52E82DE-B123-4B3E-8A7E-4FB2C6CEEE64}" name="Start" dataDxfId="8"/>
@@ -884,7 +899,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F0887D6-8664-4804-98D8-EE817E3A6A1B}">
-  <dimension ref="A1:I74"/>
+  <dimension ref="A1:I87"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -910,8 +925,8 @@
         <v>11</v>
       </c>
       <c r="D4" s="7">
-        <f>SUM(G7:G71)</f>
-        <v>7.3513888888888888</v>
+        <f>SUM(G7:G78)</f>
+        <v>8.0201388888888889</v>
       </c>
       <c r="I4" s="2"/>
     </row>
@@ -2072,7 +2087,7 @@
         <v>85</v>
       </c>
       <c r="G66" s="2">
-        <f>IF(D66&lt;C66, D66+1, D66) - C66</f>
+        <f t="shared" ref="G66:G71" si="8">IF(D66&lt;C66, D66+1, D66) - C66</f>
         <v>0.13819444444444451</v>
       </c>
     </row>
@@ -2088,7 +2103,7 @@
         <v>86</v>
       </c>
       <c r="G67" s="2">
-        <f>IF(D67&lt;C67, D67+1, D67) - C67</f>
+        <f t="shared" si="8"/>
         <v>4.8611111111111049E-2</v>
       </c>
     </row>
@@ -2107,7 +2122,7 @@
         <v>87</v>
       </c>
       <c r="G68" s="2">
-        <f>IF(D68&lt;C68, D68+1, D68) - C68</f>
+        <f t="shared" si="8"/>
         <v>9.027777777777779E-2</v>
       </c>
     </row>
@@ -2128,7 +2143,7 @@
         <v>89</v>
       </c>
       <c r="G69" s="2">
-        <f>IF(D69&lt;C69, D69+1, D69) - C69</f>
+        <f t="shared" si="8"/>
         <v>8.5416666666666696E-2</v>
       </c>
     </row>
@@ -2147,7 +2162,7 @@
         <v>90</v>
       </c>
       <c r="G70" s="2">
-        <f>IF(D70&lt;C70, D70+1, D70) - C70</f>
+        <f t="shared" si="8"/>
         <v>0.22777777777777763</v>
       </c>
     </row>
@@ -2158,7 +2173,9 @@
       <c r="C71" s="2">
         <v>0.40972222222222221</v>
       </c>
-      <c r="D71" s="2"/>
+      <c r="D71" s="2">
+        <v>0.44097222222222221</v>
+      </c>
       <c r="E71" t="s">
         <v>88</v>
       </c>
@@ -2166,22 +2183,140 @@
         <v>91</v>
       </c>
       <c r="G71" s="2">
-        <f>IF(D71&lt;C71, D71+1, D71) - C71</f>
-        <v>0.59027777777777779</v>
+        <f t="shared" si="8"/>
+        <v>3.125E-2</v>
       </c>
     </row>
     <row r="72" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="C72" s="2"/>
-      <c r="D72" s="2"/>
-      <c r="G72" s="2"/>
+      <c r="C72" s="2">
+        <v>0.44097222222222221</v>
+      </c>
+      <c r="D72" s="2">
+        <v>0.625</v>
+      </c>
+      <c r="E72" t="s">
+        <v>71</v>
+      </c>
+      <c r="F72" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="G72" s="2">
+        <f>IF(D72&lt;C72, D72+1, D72) - C72</f>
+        <v>0.18402777777777779</v>
+      </c>
     </row>
     <row r="73" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="F73" s="8" t="s">
+      <c r="C73" s="2">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="D73" s="2">
+        <v>0.77500000000000002</v>
+      </c>
+      <c r="E73" t="s">
+        <v>74</v>
+      </c>
+      <c r="F73" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="G73" s="2">
+        <f>IF(D73&lt;C73, D73+1, D73) - C73</f>
+        <v>0.10833333333333339</v>
+      </c>
+    </row>
+    <row r="74" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C74" s="2">
+        <v>0.875</v>
+      </c>
+      <c r="D74" s="2">
+        <v>0.95833333333333337</v>
+      </c>
+      <c r="E74" t="s">
+        <v>74</v>
+      </c>
+      <c r="F74" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="G74" s="2">
+        <f>IF(D74&lt;C74, D74+1, D74) - C74</f>
+        <v>8.333333333333337E-2</v>
+      </c>
+    </row>
+    <row r="75" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C75" s="2">
+        <v>0.99930555555555556</v>
+      </c>
+      <c r="D75" s="2">
+        <v>9.4444444444444442E-2</v>
+      </c>
+      <c r="E75" t="s">
+        <v>74</v>
+      </c>
+      <c r="F75" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="G75" s="2">
+        <f>IF(D75&lt;C75, D75+1, D75) - C75</f>
+        <v>9.5138888888888995E-2</v>
+      </c>
+    </row>
+    <row r="76" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B76" s="1">
+        <v>45769</v>
+      </c>
+      <c r="C76" s="2">
+        <v>0.61041666666666672</v>
+      </c>
+      <c r="D76" s="2">
+        <v>0.91666666666666663</v>
+      </c>
+      <c r="E76" t="s">
+        <v>74</v>
+      </c>
+      <c r="F76" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="G76" s="2">
+        <f>IF(D76&lt;C76, D76+1, D76) - C76</f>
+        <v>0.30624999999999991</v>
+      </c>
+    </row>
+    <row r="77" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C77" s="2">
+        <v>0.97916666666666663</v>
+      </c>
+      <c r="D77" s="2">
+        <v>6.25E-2</v>
+      </c>
+      <c r="F77" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="G77" s="2">
+        <f>IF(D77&lt;C77, D77+1, D77) - C77</f>
+        <v>8.333333333333337E-2</v>
+      </c>
+    </row>
+    <row r="78" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B78" s="1">
+        <v>45770</v>
+      </c>
+      <c r="C78" s="2">
+        <v>0.63263888888888886</v>
+      </c>
+      <c r="F78" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="G78" s="2">
+        <f>IF(D78&lt;C78, D78+1, D78) - C78</f>
+        <v>0.36736111111111114</v>
+      </c>
+    </row>
+    <row r="86" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F86" s="8" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="74" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="F74" s="9" t="s">
+    <row r="87" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F87" s="9" t="s">
         <v>42</v>
       </c>
     </row>

</xml_diff>